<commit_message>
Exclude culvert extension through the building; add culvert plan
The culvert zone now includes its extension through the building: the two
long S-SYMPOLS lines running south from the culvert, closed by the
break-line polylines at each end. Adds culvert_plan.py (plan of the zone
over the DXF) and regenerates the 1113 and 1114.85 excavation outputs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/average_levels_1113.xlsx
+++ b/average_levels_1113.xlsx
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2948.89</v>
+        <v>2581.02</v>
       </c>
     </row>
     <row r="4">
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16728.7</v>
+        <v>15794.1</v>
       </c>
     </row>
     <row r="5">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.58</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="6">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16728.12</v>
+        <v>15794.01</v>
       </c>
     </row>
     <row r="7">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>369</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2.9</v>
+        <v>370.77</v>
       </c>
     </row>
     <row r="11">
@@ -3023,7 +3023,7 @@
         <v>1113.64</v>
       </c>
       <c r="G55" t="n">
-        <v>0.13</v>
+        <v>0.01</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
@@ -3044,7 +3044,7 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0.13</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="56">
@@ -3067,7 +3067,7 @@
         <v>1111.6</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="H56" s="4" t="n">
         <v>1</v>
@@ -3088,7 +3088,7 @@
         <v>0</v>
       </c>
       <c r="N56" s="4" t="n">
-        <v>0.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -3111,7 +3111,7 @@
         <v>1115.55</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>5.25</v>
+        <v>0.51</v>
       </c>
       <c r="H57" s="4" t="n">
         <v>2</v>
@@ -3129,7 +3129,7 @@
         <v>2.045</v>
       </c>
       <c r="M57" s="4" t="n">
-        <v>10.73</v>
+        <v>1.05</v>
       </c>
       <c r="N57" s="4" t="n">
         <v>0</v>
@@ -3155,7 +3155,7 @@
         <v>1115.55</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>9</v>
+        <v>8.98</v>
       </c>
       <c r="H58" s="4" t="n">
         <v>2</v>
@@ -3173,7 +3173,7 @@
         <v>2.682</v>
       </c>
       <c r="M58" s="4" t="n">
-        <v>24.14</v>
+        <v>24.09</v>
       </c>
       <c r="N58" s="4" t="n">
         <v>0</v>
@@ -3947,7 +3947,7 @@
         <v>1115.55</v>
       </c>
       <c r="G76" s="4" t="n">
-        <v>8.789999999999999</v>
+        <v>5.68</v>
       </c>
       <c r="H76" s="4" t="n">
         <v>2</v>
@@ -3965,7 +3965,7 @@
         <v>1.085</v>
       </c>
       <c r="M76" s="4" t="n">
-        <v>9.539999999999999</v>
+        <v>6.16</v>
       </c>
       <c r="N76" s="4" t="n">
         <v>0</v>
@@ -3991,7 +3991,7 @@
         <v>1115.55</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H77" s="4" t="n">
         <v>3</v>
@@ -4009,7 +4009,7 @@
         <v>1.562</v>
       </c>
       <c r="M77" s="4" t="n">
-        <v>14.05</v>
+        <v>0</v>
       </c>
       <c r="N77" s="4" t="n">
         <v>0</v>
@@ -4035,7 +4035,7 @@
         <v>1115.55</v>
       </c>
       <c r="G78" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H78" s="4" t="n">
         <v>4</v>
@@ -4053,7 +4053,7 @@
         <v>2.55</v>
       </c>
       <c r="M78" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N78" s="4" t="n">
         <v>0</v>
@@ -4079,7 +4079,7 @@
         <v>1115.55</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>9</v>
+        <v>7.73</v>
       </c>
       <c r="H79" s="4" t="n">
         <v>4</v>
@@ -4097,7 +4097,7 @@
         <v>2.55</v>
       </c>
       <c r="M79" s="4" t="n">
-        <v>22.95</v>
+        <v>19.72</v>
       </c>
       <c r="N79" s="4" t="n">
         <v>0</v>
@@ -4827,7 +4827,7 @@
         <v>1115.55</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>9</v>
+        <v>7.83</v>
       </c>
       <c r="H96" s="4" t="n">
         <v>4</v>
@@ -4845,7 +4845,7 @@
         <v>2.55</v>
       </c>
       <c r="M96" s="4" t="n">
-        <v>22.95</v>
+        <v>19.97</v>
       </c>
       <c r="N96" s="4" t="n">
         <v>0</v>
@@ -4871,7 +4871,7 @@
         <v>1115.55</v>
       </c>
       <c r="G97" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H97" s="4" t="n">
         <v>4</v>
@@ -4889,7 +4889,7 @@
         <v>2.55</v>
       </c>
       <c r="M97" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N97" s="4" t="n">
         <v>0</v>
@@ -4915,7 +4915,7 @@
         <v>1115.55</v>
       </c>
       <c r="G98" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H98" s="4" t="n">
         <v>4</v>
@@ -4933,7 +4933,7 @@
         <v>2.55</v>
       </c>
       <c r="M98" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N98" s="4" t="n">
         <v>0</v>
@@ -4959,7 +4959,7 @@
         <v>1115.55</v>
       </c>
       <c r="G99" s="4" t="n">
-        <v>9</v>
+        <v>5.75</v>
       </c>
       <c r="H99" s="4" t="n">
         <v>4</v>
@@ -4977,7 +4977,7 @@
         <v>2.55</v>
       </c>
       <c r="M99" s="4" t="n">
-        <v>22.95</v>
+        <v>14.67</v>
       </c>
       <c r="N99" s="4" t="n">
         <v>0</v>
@@ -5707,7 +5707,7 @@
         <v>1113.39</v>
       </c>
       <c r="G116" s="4" t="n">
-        <v>9</v>
+        <v>8.99</v>
       </c>
       <c r="H116" s="4" t="n">
         <v>3</v>
@@ -5725,7 +5725,7 @@
         <v>2.01</v>
       </c>
       <c r="M116" s="4" t="n">
-        <v>18.09</v>
+        <v>18.07</v>
       </c>
       <c r="N116" s="4" t="n">
         <v>0</v>
@@ -5751,7 +5751,7 @@
         <v>1115.55</v>
       </c>
       <c r="G117" s="4" t="n">
-        <v>9</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H117" s="4" t="n">
         <v>4</v>
@@ -5769,7 +5769,7 @@
         <v>2.55</v>
       </c>
       <c r="M117" s="4" t="n">
-        <v>22.95</v>
+        <v>2.07</v>
       </c>
       <c r="N117" s="4" t="n">
         <v>0</v>
@@ -5795,7 +5795,7 @@
         <v>1115.55</v>
       </c>
       <c r="G118" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H118" s="4" t="n">
         <v>4</v>
@@ -5813,7 +5813,7 @@
         <v>2.55</v>
       </c>
       <c r="M118" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N118" s="4" t="n">
         <v>0</v>
@@ -5839,7 +5839,7 @@
         <v>1115.55</v>
       </c>
       <c r="G119" s="4" t="n">
-        <v>9</v>
+        <v>3.78</v>
       </c>
       <c r="H119" s="4" t="n">
         <v>4</v>
@@ -5857,7 +5857,7 @@
         <v>2.55</v>
       </c>
       <c r="M119" s="4" t="n">
-        <v>22.95</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="N119" s="4" t="n">
         <v>0</v>
@@ -6631,7 +6631,7 @@
         <v>1115.55</v>
       </c>
       <c r="G137" s="4" t="n">
-        <v>9</v>
+        <v>2.78</v>
       </c>
       <c r="H137" s="4" t="n">
         <v>4</v>
@@ -6649,7 +6649,7 @@
         <v>2.55</v>
       </c>
       <c r="M137" s="4" t="n">
-        <v>22.95</v>
+        <v>7.08</v>
       </c>
       <c r="N137" s="4" t="n">
         <v>0</v>
@@ -6675,7 +6675,7 @@
         <v>1115.55</v>
       </c>
       <c r="G138" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H138" s="4" t="n">
         <v>4</v>
@@ -6693,7 +6693,7 @@
         <v>2.55</v>
       </c>
       <c r="M138" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N138" s="4" t="n">
         <v>0</v>
@@ -6719,7 +6719,7 @@
         <v>1115.55</v>
       </c>
       <c r="G139" s="4" t="n">
-        <v>9</v>
+        <v>1.8</v>
       </c>
       <c r="H139" s="4" t="n">
         <v>4</v>
@@ -6737,7 +6737,7 @@
         <v>2.55</v>
       </c>
       <c r="M139" s="4" t="n">
-        <v>22.95</v>
+        <v>4.58</v>
       </c>
       <c r="N139" s="4" t="n">
         <v>0</v>
@@ -7511,7 +7511,7 @@
         <v>1115.55</v>
       </c>
       <c r="G157" s="4" t="n">
-        <v>9</v>
+        <v>4.75</v>
       </c>
       <c r="H157" s="4" t="n">
         <v>4</v>
@@ -7529,7 +7529,7 @@
         <v>2.55</v>
       </c>
       <c r="M157" s="4" t="n">
-        <v>22.95</v>
+        <v>12.11</v>
       </c>
       <c r="N157" s="4" t="n">
         <v>0</v>
@@ -7555,7 +7555,7 @@
         <v>1115.55</v>
       </c>
       <c r="G158" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H158" s="4" t="n">
         <v>4</v>
@@ -7573,7 +7573,7 @@
         <v>2.55</v>
       </c>
       <c r="M158" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N158" s="4" t="n">
         <v>0</v>
@@ -7599,7 +7599,7 @@
         <v>1115.55</v>
       </c>
       <c r="G159" s="4" t="n">
-        <v>9</v>
+        <v>0.16</v>
       </c>
       <c r="H159" s="4" t="n">
         <v>4</v>
@@ -7617,7 +7617,7 @@
         <v>2.55</v>
       </c>
       <c r="M159" s="4" t="n">
-        <v>22.95</v>
+        <v>0.42</v>
       </c>
       <c r="N159" s="4" t="n">
         <v>0</v>
@@ -7643,7 +7643,7 @@
         <v>1115.55</v>
       </c>
       <c r="G160" s="4" t="n">
-        <v>9</v>
+        <v>8.65</v>
       </c>
       <c r="H160" s="4" t="n">
         <v>4</v>
@@ -7661,7 +7661,7 @@
         <v>2.55</v>
       </c>
       <c r="M160" s="4" t="n">
-        <v>22.95</v>
+        <v>22.06</v>
       </c>
       <c r="N160" s="4" t="n">
         <v>0</v>
@@ -8391,7 +8391,7 @@
         <v>1115.55</v>
       </c>
       <c r="G177" s="4" t="n">
-        <v>9</v>
+        <v>6.72</v>
       </c>
       <c r="H177" s="4" t="n">
         <v>4</v>
@@ -8409,7 +8409,7 @@
         <v>2.55</v>
       </c>
       <c r="M177" s="4" t="n">
-        <v>22.95</v>
+        <v>17.14</v>
       </c>
       <c r="N177" s="4" t="n">
         <v>0</v>
@@ -8435,7 +8435,7 @@
         <v>1115.55</v>
       </c>
       <c r="G178" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H178" s="4" t="n">
         <v>4</v>
@@ -8453,7 +8453,7 @@
         <v>2.55</v>
       </c>
       <c r="M178" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N178" s="4" t="n">
         <v>0</v>
@@ -8479,7 +8479,7 @@
         <v>1115.55</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H179" s="4" t="n">
         <v>4</v>
@@ -8497,7 +8497,7 @@
         <v>2.55</v>
       </c>
       <c r="M179" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N179" s="4" t="n">
         <v>0</v>
@@ -8523,7 +8523,7 @@
         <v>1115.55</v>
       </c>
       <c r="G180" s="4" t="n">
-        <v>9</v>
+        <v>6.84</v>
       </c>
       <c r="H180" s="4" t="n">
         <v>4</v>
@@ -8541,7 +8541,7 @@
         <v>2.55</v>
       </c>
       <c r="M180" s="4" t="n">
-        <v>22.95</v>
+        <v>17.43</v>
       </c>
       <c r="N180" s="4" t="n">
         <v>0</v>
@@ -9183,7 +9183,7 @@
         <v>1115.55</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>9</v>
+        <v>8.58</v>
       </c>
       <c r="H195" s="4" t="n">
         <v>4</v>
@@ -9201,7 +9201,7 @@
         <v>2.55</v>
       </c>
       <c r="M195" s="4" t="n">
-        <v>22.95</v>
+        <v>21.87</v>
       </c>
       <c r="N195" s="4" t="n">
         <v>0</v>
@@ -9227,7 +9227,7 @@
         <v>1115.55</v>
       </c>
       <c r="G196" s="4" t="n">
-        <v>9</v>
+        <v>0.12</v>
       </c>
       <c r="H196" s="4" t="n">
         <v>4</v>
@@ -9245,7 +9245,7 @@
         <v>2.55</v>
       </c>
       <c r="M196" s="4" t="n">
-        <v>22.95</v>
+        <v>0.3</v>
       </c>
       <c r="N196" s="4" t="n">
         <v>0</v>
@@ -9271,7 +9271,7 @@
         <v>1115.55</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H197" s="4" t="n">
         <v>4</v>
@@ -9289,7 +9289,7 @@
         <v>2.55</v>
       </c>
       <c r="M197" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N197" s="4" t="n">
         <v>0</v>
@@ -9315,7 +9315,7 @@
         <v>1115.55</v>
       </c>
       <c r="G198" s="4" t="n">
-        <v>9</v>
+        <v>4.86</v>
       </c>
       <c r="H198" s="4" t="n">
         <v>4</v>
@@ -9333,7 +9333,7 @@
         <v>2.55</v>
       </c>
       <c r="M198" s="4" t="n">
-        <v>22.95</v>
+        <v>12.39</v>
       </c>
       <c r="N198" s="4" t="n">
         <v>0</v>
@@ -10019,7 +10019,7 @@
         <v>1115.55</v>
       </c>
       <c r="G214" s="4" t="n">
-        <v>9</v>
+        <v>1.66</v>
       </c>
       <c r="H214" s="4" t="n">
         <v>4</v>
@@ -10037,7 +10037,7 @@
         <v>2.55</v>
       </c>
       <c r="M214" s="4" t="n">
-        <v>22.95</v>
+        <v>4.24</v>
       </c>
       <c r="N214" s="4" t="n">
         <v>0</v>
@@ -10063,7 +10063,7 @@
         <v>1115.55</v>
       </c>
       <c r="G215" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H215" s="4" t="n">
         <v>4</v>
@@ -10081,7 +10081,7 @@
         <v>2.55</v>
       </c>
       <c r="M215" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N215" s="4" t="n">
         <v>0</v>
@@ -10107,7 +10107,7 @@
         <v>1115.55</v>
       </c>
       <c r="G216" s="4" t="n">
-        <v>9</v>
+        <v>2.88</v>
       </c>
       <c r="H216" s="4" t="n">
         <v>4</v>
@@ -10125,7 +10125,7 @@
         <v>2.55</v>
       </c>
       <c r="M216" s="4" t="n">
-        <v>22.95</v>
+        <v>7.34</v>
       </c>
       <c r="N216" s="4" t="n">
         <v>0</v>
@@ -10811,7 +10811,7 @@
         <v>1115.55</v>
       </c>
       <c r="G232" s="4" t="n">
-        <v>9</v>
+        <v>3.64</v>
       </c>
       <c r="H232" s="4" t="n">
         <v>4</v>
@@ -10829,7 +10829,7 @@
         <v>2.55</v>
       </c>
       <c r="M232" s="4" t="n">
-        <v>22.95</v>
+        <v>9.27</v>
       </c>
       <c r="N232" s="4" t="n">
         <v>0</v>
@@ -10855,7 +10855,7 @@
         <v>1115.55</v>
       </c>
       <c r="G233" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H233" s="4" t="n">
         <v>4</v>
@@ -10873,7 +10873,7 @@
         <v>2.55</v>
       </c>
       <c r="M233" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N233" s="4" t="n">
         <v>0</v>
@@ -10899,7 +10899,7 @@
         <v>1115.55</v>
       </c>
       <c r="G234" s="4" t="n">
-        <v>9</v>
+        <v>0.9</v>
       </c>
       <c r="H234" s="4" t="n">
         <v>4</v>
@@ -10917,7 +10917,7 @@
         <v>2.55</v>
       </c>
       <c r="M234" s="4" t="n">
-        <v>22.95</v>
+        <v>2.3</v>
       </c>
       <c r="N234" s="4" t="n">
         <v>0</v>
@@ -10961,7 +10961,7 @@
         <v>2.55</v>
       </c>
       <c r="M235" s="4" t="n">
-        <v>22.95</v>
+        <v>22.94</v>
       </c>
       <c r="N235" s="4" t="n">
         <v>0</v>
@@ -11603,7 +11603,7 @@
         <v>1115.55</v>
       </c>
       <c r="G250" s="4" t="n">
-        <v>9</v>
+        <v>5.61</v>
       </c>
       <c r="H250" s="4" t="n">
         <v>4</v>
@@ -11621,7 +11621,7 @@
         <v>2.55</v>
       </c>
       <c r="M250" s="4" t="n">
-        <v>22.95</v>
+        <v>14.3</v>
       </c>
       <c r="N250" s="4" t="n">
         <v>0</v>
@@ -11647,7 +11647,7 @@
         <v>1115.55</v>
       </c>
       <c r="G251" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H251" s="4" t="n">
         <v>4</v>
@@ -11665,7 +11665,7 @@
         <v>2.55</v>
       </c>
       <c r="M251" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N251" s="4" t="n">
         <v>0</v>
@@ -11691,7 +11691,7 @@
         <v>1115.55</v>
       </c>
       <c r="G252" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H252" s="4" t="n">
         <v>4</v>
@@ -11709,7 +11709,7 @@
         <v>2.55</v>
       </c>
       <c r="M252" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N252" s="4" t="n">
         <v>0</v>
@@ -11735,7 +11735,7 @@
         <v>1115.55</v>
       </c>
       <c r="G253" s="4" t="n">
-        <v>9</v>
+        <v>7.92</v>
       </c>
       <c r="H253" s="4" t="n">
         <v>4</v>
@@ -11753,7 +11753,7 @@
         <v>2.55</v>
       </c>
       <c r="M253" s="4" t="n">
-        <v>22.95</v>
+        <v>20.2</v>
       </c>
       <c r="N253" s="4" t="n">
         <v>0</v>
@@ -12351,7 +12351,7 @@
         <v>1121.17</v>
       </c>
       <c r="G267" s="4" t="n">
-        <v>9</v>
+        <v>7.58</v>
       </c>
       <c r="H267" s="4" t="n">
         <v>3</v>
@@ -12369,7 +12369,7 @@
         <v>3.956</v>
       </c>
       <c r="M267" s="4" t="n">
-        <v>35.6</v>
+        <v>29.99</v>
       </c>
       <c r="N267" s="4" t="n">
         <v>0</v>
@@ -12395,7 +12395,7 @@
         <v>1115.55</v>
       </c>
       <c r="G268" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H268" s="4" t="n">
         <v>4</v>
@@ -12413,7 +12413,7 @@
         <v>2.55</v>
       </c>
       <c r="M268" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N268" s="4" t="n">
         <v>0</v>
@@ -12439,7 +12439,7 @@
         <v>1115.55</v>
       </c>
       <c r="G269" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H269" s="4" t="n">
         <v>4</v>
@@ -12457,7 +12457,7 @@
         <v>2.55</v>
       </c>
       <c r="M269" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N269" s="4" t="n">
         <v>0</v>
@@ -12483,7 +12483,7 @@
         <v>1115.55</v>
       </c>
       <c r="G270" s="4" t="n">
-        <v>9</v>
+        <v>5.94</v>
       </c>
       <c r="H270" s="4" t="n">
         <v>4</v>
@@ -12501,7 +12501,7 @@
         <v>2.55</v>
       </c>
       <c r="M270" s="4" t="n">
-        <v>22.95</v>
+        <v>15.15</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>0</v>
@@ -13099,7 +13099,7 @@
         <v>1120.38</v>
       </c>
       <c r="G284" s="4" t="n">
-        <v>9</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="H284" s="4" t="n">
         <v>2</v>
@@ -13117,7 +13117,7 @@
         <v>5.164</v>
       </c>
       <c r="M284" s="4" t="n">
-        <v>46.47</v>
+        <v>46.23</v>
       </c>
       <c r="N284" s="4" t="n">
         <v>0</v>
@@ -13143,7 +13143,7 @@
         <v>1115.55</v>
       </c>
       <c r="G285" s="4" t="n">
-        <v>9</v>
+        <v>0.6</v>
       </c>
       <c r="H285" s="4" t="n">
         <v>4</v>
@@ -13161,7 +13161,7 @@
         <v>2.55</v>
       </c>
       <c r="M285" s="4" t="n">
-        <v>22.95</v>
+        <v>1.53</v>
       </c>
       <c r="N285" s="4" t="n">
         <v>0</v>
@@ -13187,7 +13187,7 @@
         <v>1115.55</v>
       </c>
       <c r="G286" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H286" s="4" t="n">
         <v>4</v>
@@ -13205,7 +13205,7 @@
         <v>2.55</v>
       </c>
       <c r="M286" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N286" s="4" t="n">
         <v>0</v>
@@ -13231,7 +13231,7 @@
         <v>1115.55</v>
       </c>
       <c r="G287" s="4" t="n">
-        <v>9</v>
+        <v>3.96</v>
       </c>
       <c r="H287" s="4" t="n">
         <v>4</v>
@@ -13249,7 +13249,7 @@
         <v>2.55</v>
       </c>
       <c r="M287" s="4" t="n">
-        <v>22.95</v>
+        <v>10.1</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>0</v>
@@ -13847,7 +13847,7 @@
         <v>1115.55</v>
       </c>
       <c r="G301" s="4" t="n">
-        <v>9</v>
+        <v>2.53</v>
       </c>
       <c r="H301" s="4" t="n">
         <v>4</v>
@@ -13865,7 +13865,7 @@
         <v>2.55</v>
       </c>
       <c r="M301" s="4" t="n">
-        <v>22.95</v>
+        <v>6.44</v>
       </c>
       <c r="N301" s="4" t="n">
         <v>0</v>
@@ -13891,7 +13891,7 @@
         <v>1115.55</v>
       </c>
       <c r="G302" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H302" s="4" t="n">
         <v>4</v>
@@ -13909,7 +13909,7 @@
         <v>2.55</v>
       </c>
       <c r="M302" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N302" s="4" t="n">
         <v>0</v>
@@ -13935,7 +13935,7 @@
         <v>1115.55</v>
       </c>
       <c r="G303" s="4" t="n">
-        <v>9</v>
+        <v>1.98</v>
       </c>
       <c r="H303" s="4" t="n">
         <v>4</v>
@@ -13953,7 +13953,7 @@
         <v>2.55</v>
       </c>
       <c r="M303" s="4" t="n">
-        <v>22.95</v>
+        <v>5.05</v>
       </c>
       <c r="N303" s="4" t="n">
         <v>0</v>
@@ -14551,7 +14551,7 @@
         <v>1115.55</v>
       </c>
       <c r="G317" s="4" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="H317" s="4" t="n">
         <v>4</v>
@@ -14569,7 +14569,7 @@
         <v>2.55</v>
       </c>
       <c r="M317" s="4" t="n">
-        <v>22.95</v>
+        <v>11.47</v>
       </c>
       <c r="N317" s="4" t="n">
         <v>0</v>
@@ -14595,7 +14595,7 @@
         <v>1115.55</v>
       </c>
       <c r="G318" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H318" s="4" t="n">
         <v>4</v>
@@ -14613,7 +14613,7 @@
         <v>2.55</v>
       </c>
       <c r="M318" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N318" s="4" t="n">
         <v>0</v>
@@ -14639,7 +14639,7 @@
         <v>1115.55</v>
       </c>
       <c r="G319" s="4" t="n">
-        <v>9</v>
+        <v>0.25</v>
       </c>
       <c r="H319" s="4" t="n">
         <v>4</v>
@@ -14657,7 +14657,7 @@
         <v>2.55</v>
       </c>
       <c r="M319" s="4" t="n">
-        <v>22.95</v>
+        <v>0.63</v>
       </c>
       <c r="N319" s="4" t="n">
         <v>0</v>
@@ -14683,7 +14683,7 @@
         <v>1115.55</v>
       </c>
       <c r="G320" s="4" t="n">
-        <v>9</v>
+        <v>8.75</v>
       </c>
       <c r="H320" s="4" t="n">
         <v>4</v>
@@ -14701,7 +14701,7 @@
         <v>2.55</v>
       </c>
       <c r="M320" s="4" t="n">
-        <v>22.95</v>
+        <v>22.32</v>
       </c>
       <c r="N320" s="4" t="n">
         <v>0</v>
@@ -15255,7 +15255,7 @@
         <v>1115.55</v>
       </c>
       <c r="G333" s="4" t="n">
-        <v>9</v>
+        <v>6.47</v>
       </c>
       <c r="H333" s="4" t="n">
         <v>4</v>
@@ -15273,7 +15273,7 @@
         <v>2.55</v>
       </c>
       <c r="M333" s="4" t="n">
-        <v>22.95</v>
+        <v>16.5</v>
       </c>
       <c r="N333" s="4" t="n">
         <v>0</v>
@@ -15299,7 +15299,7 @@
         <v>1115.55</v>
       </c>
       <c r="G334" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H334" s="4" t="n">
         <v>4</v>
@@ -15317,7 +15317,7 @@
         <v>2.55</v>
       </c>
       <c r="M334" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N334" s="4" t="n">
         <v>0</v>
@@ -15343,7 +15343,7 @@
         <v>1115.55</v>
       </c>
       <c r="G335" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H335" s="4" t="n">
         <v>4</v>
@@ -15361,7 +15361,7 @@
         <v>2.55</v>
       </c>
       <c r="M335" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N335" s="4" t="n">
         <v>0</v>
@@ -15387,7 +15387,7 @@
         <v>1115.55</v>
       </c>
       <c r="G336" s="4" t="n">
-        <v>9</v>
+        <v>7.02</v>
       </c>
       <c r="H336" s="4" t="n">
         <v>4</v>
@@ -15405,7 +15405,7 @@
         <v>2.55</v>
       </c>
       <c r="M336" s="4" t="n">
-        <v>22.95</v>
+        <v>17.91</v>
       </c>
       <c r="N336" s="4" t="n">
         <v>0</v>
@@ -15915,7 +15915,7 @@
         <v>1116.46</v>
       </c>
       <c r="G348" s="4" t="n">
-        <v>8.57</v>
+        <v>7.96</v>
       </c>
       <c r="H348" s="4" t="n">
         <v>2</v>
@@ -15933,7 +15933,7 @@
         <v>3.069</v>
       </c>
       <c r="M348" s="4" t="n">
-        <v>26.29</v>
+        <v>24.43</v>
       </c>
       <c r="N348" s="4" t="n">
         <v>0</v>
@@ -15959,7 +15959,7 @@
         <v>1116.71</v>
       </c>
       <c r="G349" s="4" t="n">
-        <v>9</v>
+        <v>0.05</v>
       </c>
       <c r="H349" s="4" t="n">
         <v>2</v>
@@ -15977,7 +15977,7 @@
         <v>3.115</v>
       </c>
       <c r="M349" s="4" t="n">
-        <v>28.03</v>
+        <v>0.15</v>
       </c>
       <c r="N349" s="4" t="n">
         <v>0</v>
@@ -16003,7 +16003,7 @@
         <v>1116.65</v>
       </c>
       <c r="G350" s="4" t="n">
-        <v>8.9</v>
+        <v>0</v>
       </c>
       <c r="H350" s="4" t="n">
         <v>2</v>
@@ -16021,7 +16021,7 @@
         <v>2.974</v>
       </c>
       <c r="M350" s="4" t="n">
-        <v>26.47</v>
+        <v>0</v>
       </c>
       <c r="N350" s="4" t="n">
         <v>0</v>
@@ -16047,7 +16047,7 @@
         <v>1116.15</v>
       </c>
       <c r="G351" s="4" t="n">
-        <v>7.61</v>
+        <v>4.21</v>
       </c>
       <c r="H351" s="4" t="n">
         <v>2</v>
@@ -16065,7 +16065,7 @@
         <v>3.325</v>
       </c>
       <c r="M351" s="4" t="n">
-        <v>25.32</v>
+        <v>13.98</v>
       </c>
       <c r="N351" s="4" t="n">
         <v>0</v>
@@ -16531,7 +16531,7 @@
         <v>1118.38</v>
       </c>
       <c r="G362" t="n">
-        <v>1.96</v>
+        <v>0.22</v>
       </c>
       <c r="H362" t="n">
         <v>0</v>
@@ -16549,7 +16549,7 @@
         <v>4.635</v>
       </c>
       <c r="M362" t="n">
-        <v>9.06</v>
+        <v>1.01</v>
       </c>
       <c r="N362" t="n">
         <v>0</v>
@@ -16575,7 +16575,7 @@
         <v>1118.8</v>
       </c>
       <c r="G363" t="n">
-        <v>0.36</v>
+        <v>0</v>
       </c>
       <c r="H363" t="n">
         <v>0</v>
@@ -16593,7 +16593,7 @@
         <v>4.712</v>
       </c>
       <c r="M363" t="n">
-        <v>1.71</v>
+        <v>0</v>
       </c>
       <c r="N363" t="n">
         <v>0</v>
@@ -17056,7 +17056,7 @@
         </is>
       </c>
       <c r="B376" t="n">
-        <v>16728.7</v>
+        <v>15794.1</v>
       </c>
     </row>
     <row r="377">
@@ -17066,7 +17066,7 @@
         </is>
       </c>
       <c r="B377" t="n">
-        <v>0.58</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="378">
@@ -17076,7 +17076,7 @@
         </is>
       </c>
       <c r="B378" t="n">
-        <v>2948.89</v>
+        <v>2581.02</v>
       </c>
     </row>
     <row r="379">
@@ -17096,7 +17096,7 @@
         </is>
       </c>
       <c r="B380" t="n">
-        <v>1118.673</v>
+        <v>1119.119</v>
       </c>
     </row>
     <row r="381">

</xml_diff>

<commit_message>
Exclude hangar footprint offset 1 m all round from area 1 volumes
The hangar outline (closed blue polyline on layer 0) is offset 1 m on its
whole perimeter and subtracted from the hatched area together with the
culvert zone. Plan drawing now shows both excluded zones.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/average_levels_1113.xlsx
+++ b/average_levels_1113.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2581.02</v>
+        <v>1690.92</v>
       </c>
     </row>
     <row r="4">
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15794.1</v>
+        <v>12976.86</v>
       </c>
     </row>
     <row r="5">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="6">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15794.01</v>
+        <v>12976.78</v>
       </c>
     </row>
     <row r="7">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>346</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -560,10 +560,30 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
+          <t>Hangar + 1 m area excluded (m²)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1260.87</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Total excluded (culvert + hangar, overlap counted once) (m²)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1260.87</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
           <t>Hangar area</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Unlabeled grid points under the hangar taken as 1115.55</t>
         </is>
@@ -632,7 +652,7 @@
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Area inside hatch excl. culvert (m²)</t>
+          <t>Area inside hatch excl. culvert &amp; hangar (m²)</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
@@ -2275,7 +2295,7 @@
         <v>1113.17</v>
       </c>
       <c r="G38" t="n">
-        <v>0.1</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -2293,7 +2313,7 @@
         <v>0.189</v>
       </c>
       <c r="M38" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="N38" t="n">
         <v>0</v>
@@ -2319,7 +2339,7 @@
         <v>1115.91</v>
       </c>
       <c r="G39" t="n">
-        <v>8.85</v>
+        <v>7.15</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -2337,7 +2357,7 @@
         <v>2.63</v>
       </c>
       <c r="M39" t="n">
-        <v>23.28</v>
+        <v>18.8</v>
       </c>
       <c r="N39" t="n">
         <v>0</v>
@@ -2363,7 +2383,7 @@
         <v>1115.72</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>9</v>
+        <v>5.37</v>
       </c>
       <c r="H40" s="4" t="n">
         <v>1</v>
@@ -2381,7 +2401,7 @@
         <v>2.603</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>23.43</v>
+        <v>13.99</v>
       </c>
       <c r="N40" s="4" t="n">
         <v>0</v>
@@ -2407,7 +2427,7 @@
         <v>1115.55</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>9</v>
+        <v>3.45</v>
       </c>
       <c r="H41" s="4" t="n">
         <v>2</v>
@@ -2425,7 +2445,7 @@
         <v>2.566</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>23.1</v>
+        <v>8.84</v>
       </c>
       <c r="N41" s="4" t="n">
         <v>0</v>
@@ -2451,7 +2471,7 @@
         <v>1115.55</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>9</v>
+        <v>1.52</v>
       </c>
       <c r="H42" s="4" t="n">
         <v>1</v>
@@ -2469,7 +2489,7 @@
         <v>3.149</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>28.35</v>
+        <v>4.78</v>
       </c>
       <c r="N42" s="4" t="n">
         <v>0</v>
@@ -2495,7 +2515,7 @@
         <v>1117.13</v>
       </c>
       <c r="G43" t="n">
-        <v>9</v>
+        <v>6.01</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -2513,7 +2533,7 @@
         <v>3.96</v>
       </c>
       <c r="M43" t="n">
-        <v>35.64</v>
+        <v>23.81</v>
       </c>
       <c r="N43" t="n">
         <v>0</v>
@@ -3023,7 +3043,7 @@
         <v>1113.64</v>
       </c>
       <c r="G55" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
@@ -3044,7 +3064,7 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -3111,7 +3131,7 @@
         <v>1115.55</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="H57" s="4" t="n">
         <v>2</v>
@@ -3129,7 +3149,7 @@
         <v>2.045</v>
       </c>
       <c r="M57" s="4" t="n">
-        <v>1.05</v>
+        <v>0</v>
       </c>
       <c r="N57" s="4" t="n">
         <v>0</v>
@@ -3155,7 +3175,7 @@
         <v>1115.55</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>8.98</v>
+        <v>0</v>
       </c>
       <c r="H58" s="4" t="n">
         <v>2</v>
@@ -3173,7 +3193,7 @@
         <v>2.682</v>
       </c>
       <c r="M58" s="4" t="n">
-        <v>24.09</v>
+        <v>0</v>
       </c>
       <c r="N58" s="4" t="n">
         <v>0</v>
@@ -3199,7 +3219,7 @@
         <v>1115.55</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H59" s="4" t="n">
         <v>3</v>
@@ -3217,7 +3237,7 @@
         <v>2.592</v>
       </c>
       <c r="M59" s="4" t="n">
-        <v>23.33</v>
+        <v>0</v>
       </c>
       <c r="N59" s="4" t="n">
         <v>0</v>
@@ -3243,7 +3263,7 @@
         <v>1115.55</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H60" s="4" t="n">
         <v>4</v>
@@ -3261,7 +3281,7 @@
         <v>2.55</v>
       </c>
       <c r="M60" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N60" s="4" t="n">
         <v>0</v>
@@ -3287,7 +3307,7 @@
         <v>1115.55</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H61" s="4" t="n">
         <v>3</v>
@@ -3305,7 +3325,7 @@
         <v>2.945</v>
       </c>
       <c r="M61" s="4" t="n">
-        <v>26.5</v>
+        <v>0</v>
       </c>
       <c r="N61" s="4" t="n">
         <v>0</v>
@@ -3331,7 +3351,7 @@
         <v>1115.55</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>9</v>
+        <v>4.02</v>
       </c>
       <c r="H62" s="4" t="n">
         <v>1</v>
@@ -3349,7 +3369,7 @@
         <v>3.999</v>
       </c>
       <c r="M62" s="4" t="n">
-        <v>35.99</v>
+        <v>16.07</v>
       </c>
       <c r="N62" s="4" t="n">
         <v>0</v>
@@ -3903,7 +3923,7 @@
         <v>1112.26</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>7.17</v>
+        <v>2.25</v>
       </c>
       <c r="H75" s="4" t="n">
         <v>1</v>
@@ -3921,7 +3941,7 @@
         <v>0.367</v>
       </c>
       <c r="M75" s="4" t="n">
-        <v>2.63</v>
+        <v>0.82</v>
       </c>
       <c r="N75" s="4" t="n">
         <v>0</v>
@@ -3947,7 +3967,7 @@
         <v>1115.55</v>
       </c>
       <c r="G76" s="4" t="n">
-        <v>5.68</v>
+        <v>0</v>
       </c>
       <c r="H76" s="4" t="n">
         <v>2</v>
@@ -3965,7 +3985,7 @@
         <v>1.085</v>
       </c>
       <c r="M76" s="4" t="n">
-        <v>6.16</v>
+        <v>0</v>
       </c>
       <c r="N76" s="4" t="n">
         <v>0</v>
@@ -4079,7 +4099,7 @@
         <v>1115.55</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>7.73</v>
+        <v>0</v>
       </c>
       <c r="H79" s="4" t="n">
         <v>4</v>
@@ -4097,7 +4117,7 @@
         <v>2.55</v>
       </c>
       <c r="M79" s="4" t="n">
-        <v>19.72</v>
+        <v>0</v>
       </c>
       <c r="N79" s="4" t="n">
         <v>0</v>
@@ -4123,7 +4143,7 @@
         <v>1115.55</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H80" s="4" t="n">
         <v>4</v>
@@ -4141,7 +4161,7 @@
         <v>2.55</v>
       </c>
       <c r="M80" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N80" s="4" t="n">
         <v>0</v>
@@ -4167,7 +4187,7 @@
         <v>1115.55</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H81" s="4" t="n">
         <v>4</v>
@@ -4185,7 +4205,7 @@
         <v>2.55</v>
       </c>
       <c r="M81" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N81" s="4" t="n">
         <v>0</v>
@@ -4211,7 +4231,7 @@
         <v>1115.55</v>
       </c>
       <c r="G82" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H82" s="4" t="n">
         <v>4</v>
@@ -4229,7 +4249,7 @@
         <v>2.55</v>
       </c>
       <c r="M82" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N82" s="4" t="n">
         <v>0</v>
@@ -4255,7 +4275,7 @@
         <v>1115.55</v>
       </c>
       <c r="G83" s="4" t="n">
-        <v>9</v>
+        <v>2.1</v>
       </c>
       <c r="H83" s="4" t="n">
         <v>2</v>
@@ -4273,7 +4293,7 @@
         <v>3.949</v>
       </c>
       <c r="M83" s="4" t="n">
-        <v>35.54</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N83" s="4" t="n">
         <v>0</v>
@@ -4783,7 +4803,7 @@
         <v>1112.56</v>
       </c>
       <c r="G95" s="4" t="n">
-        <v>7.32</v>
+        <v>3.23</v>
       </c>
       <c r="H95" s="4" t="n">
         <v>2</v>
@@ -4801,7 +4821,7 @@
         <v>0.98</v>
       </c>
       <c r="M95" s="4" t="n">
-        <v>7.17</v>
+        <v>3.17</v>
       </c>
       <c r="N95" s="4" t="n">
         <v>0</v>
@@ -4827,7 +4847,7 @@
         <v>1115.55</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>7.83</v>
+        <v>0</v>
       </c>
       <c r="H96" s="4" t="n">
         <v>4</v>
@@ -4845,7 +4865,7 @@
         <v>2.55</v>
       </c>
       <c r="M96" s="4" t="n">
-        <v>19.97</v>
+        <v>0</v>
       </c>
       <c r="N96" s="4" t="n">
         <v>0</v>
@@ -4959,7 +4979,7 @@
         <v>1115.55</v>
       </c>
       <c r="G99" s="4" t="n">
-        <v>5.75</v>
+        <v>0</v>
       </c>
       <c r="H99" s="4" t="n">
         <v>4</v>
@@ -4977,7 +4997,7 @@
         <v>2.55</v>
       </c>
       <c r="M99" s="4" t="n">
-        <v>14.67</v>
+        <v>0</v>
       </c>
       <c r="N99" s="4" t="n">
         <v>0</v>
@@ -5003,7 +5023,7 @@
         <v>1115.55</v>
       </c>
       <c r="G100" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H100" s="4" t="n">
         <v>4</v>
@@ -5021,7 +5041,7 @@
         <v>2.55</v>
       </c>
       <c r="M100" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N100" s="4" t="n">
         <v>0</v>
@@ -5047,7 +5067,7 @@
         <v>1115.55</v>
       </c>
       <c r="G101" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H101" s="4" t="n">
         <v>4</v>
@@ -5065,7 +5085,7 @@
         <v>2.55</v>
       </c>
       <c r="M101" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N101" s="4" t="n">
         <v>0</v>
@@ -5091,7 +5111,7 @@
         <v>1115.55</v>
       </c>
       <c r="G102" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H102" s="4" t="n">
         <v>4</v>
@@ -5109,7 +5129,7 @@
         <v>2.55</v>
       </c>
       <c r="M102" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N102" s="4" t="n">
         <v>0</v>
@@ -5135,7 +5155,7 @@
         <v>1115.55</v>
       </c>
       <c r="G103" s="4" t="n">
-        <v>9</v>
+        <v>0.34</v>
       </c>
       <c r="H103" s="4" t="n">
         <v>2</v>
@@ -5153,7 +5173,7 @@
         <v>4.007</v>
       </c>
       <c r="M103" s="4" t="n">
-        <v>36.07</v>
+        <v>1.36</v>
       </c>
       <c r="N103" s="4" t="n">
         <v>0</v>
@@ -5179,7 +5199,7 @@
         <v>1118.12</v>
       </c>
       <c r="G104" t="n">
-        <v>9</v>
+        <v>8.84</v>
       </c>
       <c r="H104" t="n">
         <v>0</v>
@@ -5197,7 +5217,7 @@
         <v>6.025</v>
       </c>
       <c r="M104" t="n">
-        <v>54.23</v>
+        <v>53.28</v>
       </c>
       <c r="N104" t="n">
         <v>0</v>
@@ -5663,7 +5683,7 @@
         <v>1112.87</v>
       </c>
       <c r="G115" s="4" t="n">
-        <v>5.48</v>
+        <v>3.3</v>
       </c>
       <c r="H115" s="4" t="n">
         <v>1</v>
@@ -5681,7 +5701,7 @@
         <v>0.592</v>
       </c>
       <c r="M115" s="4" t="n">
-        <v>3.24</v>
+        <v>1.96</v>
       </c>
       <c r="N115" s="4" t="n">
         <v>0</v>
@@ -5707,7 +5727,7 @@
         <v>1113.39</v>
       </c>
       <c r="G116" s="4" t="n">
-        <v>8.99</v>
+        <v>0</v>
       </c>
       <c r="H116" s="4" t="n">
         <v>3</v>
@@ -5725,7 +5745,7 @@
         <v>2.01</v>
       </c>
       <c r="M116" s="4" t="n">
-        <v>18.07</v>
+        <v>0</v>
       </c>
       <c r="N116" s="4" t="n">
         <v>0</v>
@@ -5751,7 +5771,7 @@
         <v>1115.55</v>
       </c>
       <c r="G117" s="4" t="n">
-        <v>0.8100000000000001</v>
+        <v>0</v>
       </c>
       <c r="H117" s="4" t="n">
         <v>4</v>
@@ -5769,7 +5789,7 @@
         <v>2.55</v>
       </c>
       <c r="M117" s="4" t="n">
-        <v>2.07</v>
+        <v>0</v>
       </c>
       <c r="N117" s="4" t="n">
         <v>0</v>
@@ -5839,7 +5859,7 @@
         <v>1115.55</v>
       </c>
       <c r="G119" s="4" t="n">
-        <v>3.78</v>
+        <v>0</v>
       </c>
       <c r="H119" s="4" t="n">
         <v>4</v>
@@ -5857,7 +5877,7 @@
         <v>2.55</v>
       </c>
       <c r="M119" s="4" t="n">
-        <v>9.630000000000001</v>
+        <v>0</v>
       </c>
       <c r="N119" s="4" t="n">
         <v>0</v>
@@ -5883,7 +5903,7 @@
         <v>1115.55</v>
       </c>
       <c r="G120" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H120" s="4" t="n">
         <v>4</v>
@@ -5901,7 +5921,7 @@
         <v>2.55</v>
       </c>
       <c r="M120" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N120" s="4" t="n">
         <v>0</v>
@@ -5927,7 +5947,7 @@
         <v>1115.55</v>
       </c>
       <c r="G121" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H121" s="4" t="n">
         <v>4</v>
@@ -5945,7 +5965,7 @@
         <v>2.55</v>
       </c>
       <c r="M121" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N121" s="4" t="n">
         <v>0</v>
@@ -5971,7 +5991,7 @@
         <v>1115.55</v>
       </c>
       <c r="G122" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H122" s="4" t="n">
         <v>4</v>
@@ -5989,7 +6009,7 @@
         <v>2.55</v>
       </c>
       <c r="M122" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N122" s="4" t="n">
         <v>0</v>
@@ -6015,7 +6035,7 @@
         <v>1115.55</v>
       </c>
       <c r="G123" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H123" s="4" t="n">
         <v>2</v>
@@ -6033,7 +6053,7 @@
         <v>3.84</v>
       </c>
       <c r="M123" s="4" t="n">
-        <v>34.56</v>
+        <v>0</v>
       </c>
       <c r="N123" s="4" t="n">
         <v>0</v>
@@ -6059,7 +6079,7 @@
         <v>1118.14</v>
       </c>
       <c r="G124" t="n">
-        <v>9</v>
+        <v>7.26</v>
       </c>
       <c r="H124" t="n">
         <v>0</v>
@@ -6077,7 +6097,7 @@
         <v>5.731</v>
       </c>
       <c r="M124" t="n">
-        <v>51.58</v>
+        <v>41.63</v>
       </c>
       <c r="N124" t="n">
         <v>0</v>
@@ -6543,7 +6563,7 @@
         <v>1113.14</v>
       </c>
       <c r="G135" t="n">
-        <v>3.64</v>
+        <v>3.25</v>
       </c>
       <c r="H135" t="n">
         <v>0</v>
@@ -6561,7 +6581,7 @@
         <v>0.215</v>
       </c>
       <c r="M135" t="n">
-        <v>0.78</v>
+        <v>0.7</v>
       </c>
       <c r="N135" t="n">
         <v>0</v>
@@ -6587,7 +6607,7 @@
         <v>1113.47</v>
       </c>
       <c r="G136" s="4" t="n">
-        <v>9</v>
+        <v>0.13</v>
       </c>
       <c r="H136" s="4" t="n">
         <v>2</v>
@@ -6605,7 +6625,7 @@
         <v>1.489</v>
       </c>
       <c r="M136" s="4" t="n">
-        <v>13.4</v>
+        <v>0.19</v>
       </c>
       <c r="N136" s="4" t="n">
         <v>0</v>
@@ -6631,7 +6651,7 @@
         <v>1115.55</v>
       </c>
       <c r="G137" s="4" t="n">
-        <v>2.78</v>
+        <v>0</v>
       </c>
       <c r="H137" s="4" t="n">
         <v>4</v>
@@ -6649,7 +6669,7 @@
         <v>2.55</v>
       </c>
       <c r="M137" s="4" t="n">
-        <v>7.08</v>
+        <v>0</v>
       </c>
       <c r="N137" s="4" t="n">
         <v>0</v>
@@ -6719,7 +6739,7 @@
         <v>1115.55</v>
       </c>
       <c r="G139" s="4" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="H139" s="4" t="n">
         <v>4</v>
@@ -6737,7 +6757,7 @@
         <v>2.55</v>
       </c>
       <c r="M139" s="4" t="n">
-        <v>4.58</v>
+        <v>0</v>
       </c>
       <c r="N139" s="4" t="n">
         <v>0</v>
@@ -6763,7 +6783,7 @@
         <v>1115.55</v>
       </c>
       <c r="G140" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H140" s="4" t="n">
         <v>4</v>
@@ -6781,7 +6801,7 @@
         <v>2.55</v>
       </c>
       <c r="M140" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N140" s="4" t="n">
         <v>0</v>
@@ -6807,7 +6827,7 @@
         <v>1115.55</v>
       </c>
       <c r="G141" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H141" s="4" t="n">
         <v>4</v>
@@ -6825,7 +6845,7 @@
         <v>2.55</v>
       </c>
       <c r="M141" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N141" s="4" t="n">
         <v>0</v>
@@ -6851,7 +6871,7 @@
         <v>1115.55</v>
       </c>
       <c r="G142" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H142" s="4" t="n">
         <v>4</v>
@@ -6869,7 +6889,7 @@
         <v>2.55</v>
       </c>
       <c r="M142" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N142" s="4" t="n">
         <v>0</v>
@@ -6895,7 +6915,7 @@
         <v>1115.55</v>
       </c>
       <c r="G143" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H143" s="4" t="n">
         <v>2</v>
@@ -6913,7 +6933,7 @@
         <v>3.858</v>
       </c>
       <c r="M143" s="4" t="n">
-        <v>34.72</v>
+        <v>0</v>
       </c>
       <c r="N143" s="4" t="n">
         <v>0</v>
@@ -6939,7 +6959,7 @@
         <v>1118.19</v>
       </c>
       <c r="G144" t="n">
-        <v>9</v>
+        <v>5.34</v>
       </c>
       <c r="H144" t="n">
         <v>0</v>
@@ -6957,7 +6977,7 @@
         <v>5.699</v>
       </c>
       <c r="M144" t="n">
-        <v>51.29</v>
+        <v>30.45</v>
       </c>
       <c r="N144" t="n">
         <v>0</v>
@@ -7467,7 +7487,7 @@
         <v>1113.07</v>
       </c>
       <c r="G156" s="4" t="n">
-        <v>9</v>
+        <v>1.72</v>
       </c>
       <c r="H156" s="4" t="n">
         <v>2</v>
@@ -7485,7 +7505,7 @@
         <v>1.409</v>
       </c>
       <c r="M156" s="4" t="n">
-        <v>12.68</v>
+        <v>2.42</v>
       </c>
       <c r="N156" s="4" t="n">
         <v>0</v>
@@ -7511,7 +7531,7 @@
         <v>1115.55</v>
       </c>
       <c r="G157" s="4" t="n">
-        <v>4.75</v>
+        <v>0</v>
       </c>
       <c r="H157" s="4" t="n">
         <v>4</v>
@@ -7529,7 +7549,7 @@
         <v>2.55</v>
       </c>
       <c r="M157" s="4" t="n">
-        <v>12.11</v>
+        <v>0</v>
       </c>
       <c r="N157" s="4" t="n">
         <v>0</v>
@@ -7599,7 +7619,7 @@
         <v>1115.55</v>
       </c>
       <c r="G159" s="4" t="n">
-        <v>0.16</v>
+        <v>0</v>
       </c>
       <c r="H159" s="4" t="n">
         <v>4</v>
@@ -7617,7 +7637,7 @@
         <v>2.55</v>
       </c>
       <c r="M159" s="4" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="N159" s="4" t="n">
         <v>0</v>
@@ -7643,7 +7663,7 @@
         <v>1115.55</v>
       </c>
       <c r="G160" s="4" t="n">
-        <v>8.65</v>
+        <v>0</v>
       </c>
       <c r="H160" s="4" t="n">
         <v>4</v>
@@ -7661,7 +7681,7 @@
         <v>2.55</v>
       </c>
       <c r="M160" s="4" t="n">
-        <v>22.06</v>
+        <v>0</v>
       </c>
       <c r="N160" s="4" t="n">
         <v>0</v>
@@ -7687,7 +7707,7 @@
         <v>1115.55</v>
       </c>
       <c r="G161" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H161" s="4" t="n">
         <v>4</v>
@@ -7705,7 +7725,7 @@
         <v>2.55</v>
       </c>
       <c r="M161" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N161" s="4" t="n">
         <v>0</v>
@@ -7731,7 +7751,7 @@
         <v>1115.55</v>
       </c>
       <c r="G162" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H162" s="4" t="n">
         <v>4</v>
@@ -7749,7 +7769,7 @@
         <v>2.55</v>
       </c>
       <c r="M162" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N162" s="4" t="n">
         <v>0</v>
@@ -7775,7 +7795,7 @@
         <v>1115.55</v>
       </c>
       <c r="G163" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H163" s="4" t="n">
         <v>3</v>
@@ -7793,7 +7813,7 @@
         <v>3.211</v>
       </c>
       <c r="M163" s="4" t="n">
-        <v>28.9</v>
+        <v>0</v>
       </c>
       <c r="N163" s="4" t="n">
         <v>0</v>
@@ -7819,7 +7839,7 @@
         <v>1115.55</v>
       </c>
       <c r="G164" s="4" t="n">
-        <v>9</v>
+        <v>3.33</v>
       </c>
       <c r="H164" s="4" t="n">
         <v>1</v>
@@ -7837,7 +7857,7 @@
         <v>5.129</v>
       </c>
       <c r="M164" s="4" t="n">
-        <v>46.17</v>
+        <v>17.1</v>
       </c>
       <c r="N164" s="4" t="n">
         <v>0</v>
@@ -8347,7 +8367,7 @@
         <v>1113.48</v>
       </c>
       <c r="G176" s="4" t="n">
-        <v>8.74</v>
+        <v>3.46</v>
       </c>
       <c r="H176" s="4" t="n">
         <v>2</v>
@@ -8365,7 +8385,7 @@
         <v>1.413</v>
       </c>
       <c r="M176" s="4" t="n">
-        <v>12.36</v>
+        <v>4.89</v>
       </c>
       <c r="N176" s="4" t="n">
         <v>0</v>
@@ -8391,7 +8411,7 @@
         <v>1115.55</v>
       </c>
       <c r="G177" s="4" t="n">
-        <v>6.72</v>
+        <v>0</v>
       </c>
       <c r="H177" s="4" t="n">
         <v>4</v>
@@ -8409,7 +8429,7 @@
         <v>2.55</v>
       </c>
       <c r="M177" s="4" t="n">
-        <v>17.14</v>
+        <v>0</v>
       </c>
       <c r="N177" s="4" t="n">
         <v>0</v>
@@ -8523,7 +8543,7 @@
         <v>1115.55</v>
       </c>
       <c r="G180" s="4" t="n">
-        <v>6.84</v>
+        <v>0</v>
       </c>
       <c r="H180" s="4" t="n">
         <v>4</v>
@@ -8541,7 +8561,7 @@
         <v>2.55</v>
       </c>
       <c r="M180" s="4" t="n">
-        <v>17.43</v>
+        <v>0</v>
       </c>
       <c r="N180" s="4" t="n">
         <v>0</v>
@@ -8567,7 +8587,7 @@
         <v>1115.55</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H181" s="4" t="n">
         <v>4</v>
@@ -8585,7 +8605,7 @@
         <v>2.55</v>
       </c>
       <c r="M181" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N181" s="4" t="n">
         <v>0</v>
@@ -8611,7 +8631,7 @@
         <v>1115.55</v>
       </c>
       <c r="G182" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H182" s="4" t="n">
         <v>4</v>
@@ -8629,7 +8649,7 @@
         <v>2.55</v>
       </c>
       <c r="M182" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N182" s="4" t="n">
         <v>0</v>
@@ -8655,7 +8675,7 @@
         <v>1115.55</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H183" s="4" t="n">
         <v>4</v>
@@ -8673,7 +8693,7 @@
         <v>2.55</v>
       </c>
       <c r="M183" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N183" s="4" t="n">
         <v>0</v>
@@ -8699,7 +8719,7 @@
         <v>1115.55</v>
       </c>
       <c r="G184" s="4" t="n">
-        <v>9</v>
+        <v>1.28</v>
       </c>
       <c r="H184" s="4" t="n">
         <v>2</v>
@@ -8717,7 +8737,7 @@
         <v>4.217</v>
       </c>
       <c r="M184" s="4" t="n">
-        <v>37.96</v>
+        <v>5.4</v>
       </c>
       <c r="N184" s="4" t="n">
         <v>0</v>
@@ -9139,7 +9159,7 @@
         <v>1113.9</v>
       </c>
       <c r="G194" s="4" t="n">
-        <v>7.11</v>
+        <v>3.81</v>
       </c>
       <c r="H194" s="4" t="n">
         <v>2</v>
@@ -9157,7 +9177,7 @@
         <v>1.621</v>
       </c>
       <c r="M194" s="4" t="n">
-        <v>11.52</v>
+        <v>6.19</v>
       </c>
       <c r="N194" s="4" t="n">
         <v>0</v>
@@ -9183,7 +9203,7 @@
         <v>1115.55</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>8.58</v>
+        <v>0</v>
       </c>
       <c r="H195" s="4" t="n">
         <v>4</v>
@@ -9201,7 +9221,7 @@
         <v>2.55</v>
       </c>
       <c r="M195" s="4" t="n">
-        <v>21.87</v>
+        <v>0</v>
       </c>
       <c r="N195" s="4" t="n">
         <v>0</v>
@@ -9227,7 +9247,7 @@
         <v>1115.55</v>
       </c>
       <c r="G196" s="4" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="H196" s="4" t="n">
         <v>4</v>
@@ -9245,7 +9265,7 @@
         <v>2.55</v>
       </c>
       <c r="M196" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="N196" s="4" t="n">
         <v>0</v>
@@ -9315,7 +9335,7 @@
         <v>1115.55</v>
       </c>
       <c r="G198" s="4" t="n">
-        <v>4.86</v>
+        <v>0</v>
       </c>
       <c r="H198" s="4" t="n">
         <v>4</v>
@@ -9333,7 +9353,7 @@
         <v>2.55</v>
       </c>
       <c r="M198" s="4" t="n">
-        <v>12.39</v>
+        <v>0</v>
       </c>
       <c r="N198" s="4" t="n">
         <v>0</v>
@@ -9359,7 +9379,7 @@
         <v>1115.55</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H199" s="4" t="n">
         <v>4</v>
@@ -9377,7 +9397,7 @@
         <v>2.55</v>
       </c>
       <c r="M199" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N199" s="4" t="n">
         <v>0</v>
@@ -9403,7 +9423,7 @@
         <v>1115.55</v>
       </c>
       <c r="G200" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H200" s="4" t="n">
         <v>4</v>
@@ -9421,7 +9441,7 @@
         <v>2.55</v>
       </c>
       <c r="M200" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N200" s="4" t="n">
         <v>0</v>
@@ -9447,7 +9467,7 @@
         <v>1115.55</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H201" s="4" t="n">
         <v>4</v>
@@ -9465,7 +9485,7 @@
         <v>2.55</v>
       </c>
       <c r="M201" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N201" s="4" t="n">
         <v>0</v>
@@ -9491,7 +9511,7 @@
         <v>1115.55</v>
       </c>
       <c r="G202" s="4" t="n">
-        <v>9</v>
+        <v>0.02</v>
       </c>
       <c r="H202" s="4" t="n">
         <v>2</v>
@@ -9509,7 +9529,7 @@
         <v>4.1</v>
       </c>
       <c r="M202" s="4" t="n">
-        <v>36.9</v>
+        <v>0.06</v>
       </c>
       <c r="N202" s="4" t="n">
         <v>0</v>
@@ -9535,7 +9555,7 @@
         <v>1118.66</v>
       </c>
       <c r="G203" t="n">
-        <v>9</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="H203" t="n">
         <v>0</v>
@@ -9553,7 +9573,7 @@
         <v>6.8</v>
       </c>
       <c r="M203" t="n">
-        <v>61.2</v>
+        <v>55.85</v>
       </c>
       <c r="N203" t="n">
         <v>0</v>
@@ -9931,7 +9951,7 @@
         <v>1114.04</v>
       </c>
       <c r="G212" s="4" t="n">
-        <v>5.26</v>
+        <v>3.98</v>
       </c>
       <c r="H212" s="4" t="n">
         <v>1</v>
@@ -9949,7 +9969,7 @@
         <v>1.51</v>
       </c>
       <c r="M212" s="4" t="n">
-        <v>7.95</v>
+        <v>6.02</v>
       </c>
       <c r="N212" s="4" t="n">
         <v>0</v>
@@ -9975,7 +9995,7 @@
         <v>1114.55</v>
       </c>
       <c r="G213" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H213" s="4" t="n">
         <v>3</v>
@@ -9993,7 +10013,7 @@
         <v>2.3</v>
       </c>
       <c r="M213" s="4" t="n">
-        <v>20.7</v>
+        <v>0</v>
       </c>
       <c r="N213" s="4" t="n">
         <v>0</v>
@@ -10019,7 +10039,7 @@
         <v>1115.55</v>
       </c>
       <c r="G214" s="4" t="n">
-        <v>1.66</v>
+        <v>0</v>
       </c>
       <c r="H214" s="4" t="n">
         <v>4</v>
@@ -10037,7 +10057,7 @@
         <v>2.55</v>
       </c>
       <c r="M214" s="4" t="n">
-        <v>4.24</v>
+        <v>0</v>
       </c>
       <c r="N214" s="4" t="n">
         <v>0</v>
@@ -10107,7 +10127,7 @@
         <v>1115.55</v>
       </c>
       <c r="G216" s="4" t="n">
-        <v>2.88</v>
+        <v>0</v>
       </c>
       <c r="H216" s="4" t="n">
         <v>4</v>
@@ -10125,7 +10145,7 @@
         <v>2.55</v>
       </c>
       <c r="M216" s="4" t="n">
-        <v>7.34</v>
+        <v>0</v>
       </c>
       <c r="N216" s="4" t="n">
         <v>0</v>
@@ -10151,7 +10171,7 @@
         <v>1115.55</v>
       </c>
       <c r="G217" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H217" s="4" t="n">
         <v>4</v>
@@ -10169,7 +10189,7 @@
         <v>2.55</v>
       </c>
       <c r="M217" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N217" s="4" t="n">
         <v>0</v>
@@ -10195,7 +10215,7 @@
         <v>1115.55</v>
       </c>
       <c r="G218" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H218" s="4" t="n">
         <v>4</v>
@@ -10213,7 +10233,7 @@
         <v>2.55</v>
       </c>
       <c r="M218" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N218" s="4" t="n">
         <v>0</v>
@@ -10239,7 +10259,7 @@
         <v>1115.55</v>
       </c>
       <c r="G219" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H219" s="4" t="n">
         <v>4</v>
@@ -10257,7 +10277,7 @@
         <v>2.55</v>
       </c>
       <c r="M219" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N219" s="4" t="n">
         <v>0</v>
@@ -10283,7 +10303,7 @@
         <v>1115.55</v>
       </c>
       <c r="G220" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H220" s="4" t="n">
         <v>2</v>
@@ -10301,7 +10321,7 @@
         <v>4.171</v>
       </c>
       <c r="M220" s="4" t="n">
-        <v>37.54</v>
+        <v>0</v>
       </c>
       <c r="N220" s="4" t="n">
         <v>0</v>
@@ -10327,7 +10347,7 @@
         <v>1118.93</v>
       </c>
       <c r="G221" t="n">
-        <v>9</v>
+        <v>6.18</v>
       </c>
       <c r="H221" t="n">
         <v>0</v>
@@ -10345,7 +10365,7 @@
         <v>6.505</v>
       </c>
       <c r="M221" t="n">
-        <v>58.55</v>
+        <v>40.18</v>
       </c>
       <c r="N221" t="n">
         <v>0</v>
@@ -10723,7 +10743,7 @@
         <v>1114.13</v>
       </c>
       <c r="G230" t="n">
-        <v>3.42</v>
+        <v>3.41</v>
       </c>
       <c r="H230" t="n">
         <v>0</v>
@@ -10741,7 +10761,7 @@
         <v>1.241</v>
       </c>
       <c r="M230" t="n">
-        <v>4.24</v>
+        <v>4.23</v>
       </c>
       <c r="N230" t="n">
         <v>0</v>
@@ -10767,7 +10787,7 @@
         <v>1114.24</v>
       </c>
       <c r="G231" s="4" t="n">
-        <v>9</v>
+        <v>0.88</v>
       </c>
       <c r="H231" s="4" t="n">
         <v>2</v>
@@ -10785,7 +10805,7 @@
         <v>1.973</v>
       </c>
       <c r="M231" s="4" t="n">
-        <v>17.76</v>
+        <v>1.73</v>
       </c>
       <c r="N231" s="4" t="n">
         <v>0</v>
@@ -10811,7 +10831,7 @@
         <v>1115.55</v>
       </c>
       <c r="G232" s="4" t="n">
-        <v>3.64</v>
+        <v>0</v>
       </c>
       <c r="H232" s="4" t="n">
         <v>4</v>
@@ -10829,7 +10849,7 @@
         <v>2.55</v>
       </c>
       <c r="M232" s="4" t="n">
-        <v>9.27</v>
+        <v>0</v>
       </c>
       <c r="N232" s="4" t="n">
         <v>0</v>
@@ -10899,7 +10919,7 @@
         <v>1115.55</v>
       </c>
       <c r="G234" s="4" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="H234" s="4" t="n">
         <v>4</v>
@@ -10917,7 +10937,7 @@
         <v>2.55</v>
       </c>
       <c r="M234" s="4" t="n">
-        <v>2.3</v>
+        <v>0</v>
       </c>
       <c r="N234" s="4" t="n">
         <v>0</v>
@@ -10943,7 +10963,7 @@
         <v>1115.55</v>
       </c>
       <c r="G235" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H235" s="4" t="n">
         <v>4</v>
@@ -10961,7 +10981,7 @@
         <v>2.55</v>
       </c>
       <c r="M235" s="4" t="n">
-        <v>22.94</v>
+        <v>0</v>
       </c>
       <c r="N235" s="4" t="n">
         <v>0</v>
@@ -10987,7 +11007,7 @@
         <v>1115.55</v>
       </c>
       <c r="G236" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H236" s="4" t="n">
         <v>4</v>
@@ -11005,7 +11025,7 @@
         <v>2.55</v>
       </c>
       <c r="M236" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N236" s="4" t="n">
         <v>0</v>
@@ -11031,7 +11051,7 @@
         <v>1115.55</v>
       </c>
       <c r="G237" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H237" s="4" t="n">
         <v>4</v>
@@ -11049,7 +11069,7 @@
         <v>2.55</v>
       </c>
       <c r="M237" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N237" s="4" t="n">
         <v>0</v>
@@ -11075,7 +11095,7 @@
         <v>1115.55</v>
       </c>
       <c r="G238" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H238" s="4" t="n">
         <v>2</v>
@@ -11093,7 +11113,7 @@
         <v>6.23</v>
       </c>
       <c r="M238" s="4" t="n">
-        <v>56.07</v>
+        <v>0</v>
       </c>
       <c r="N238" s="4" t="n">
         <v>0</v>
@@ -11119,7 +11139,7 @@
         <v>1126.89</v>
       </c>
       <c r="G239" t="n">
-        <v>9</v>
+        <v>4.12</v>
       </c>
       <c r="H239" t="n">
         <v>0</v>
@@ -11137,7 +11157,7 @@
         <v>9.573</v>
       </c>
       <c r="M239" t="n">
-        <v>86.16</v>
+        <v>39.49</v>
       </c>
       <c r="N239" t="n">
         <v>0</v>
@@ -11559,7 +11579,7 @@
         <v>1114.64</v>
       </c>
       <c r="G249" s="4" t="n">
-        <v>2.71</v>
+        <v>0.36</v>
       </c>
       <c r="H249" s="4" t="n">
         <v>2</v>
@@ -11577,7 +11597,7 @@
         <v>1.995</v>
       </c>
       <c r="M249" s="4" t="n">
-        <v>5.4</v>
+        <v>0.71</v>
       </c>
       <c r="N249" s="4" t="n">
         <v>0</v>
@@ -11603,7 +11623,7 @@
         <v>1115.55</v>
       </c>
       <c r="G250" s="4" t="n">
-        <v>5.61</v>
+        <v>0</v>
       </c>
       <c r="H250" s="4" t="n">
         <v>4</v>
@@ -11621,7 +11641,7 @@
         <v>2.55</v>
       </c>
       <c r="M250" s="4" t="n">
-        <v>14.3</v>
+        <v>0</v>
       </c>
       <c r="N250" s="4" t="n">
         <v>0</v>
@@ -11735,7 +11755,7 @@
         <v>1115.55</v>
       </c>
       <c r="G253" s="4" t="n">
-        <v>7.92</v>
+        <v>0</v>
       </c>
       <c r="H253" s="4" t="n">
         <v>4</v>
@@ -11753,7 +11773,7 @@
         <v>2.55</v>
       </c>
       <c r="M253" s="4" t="n">
-        <v>20.2</v>
+        <v>0</v>
       </c>
       <c r="N253" s="4" t="n">
         <v>0</v>
@@ -11779,7 +11799,7 @@
         <v>1115.55</v>
       </c>
       <c r="G254" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H254" s="4" t="n">
         <v>4</v>
@@ -11797,7 +11817,7 @@
         <v>2.55</v>
       </c>
       <c r="M254" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N254" s="4" t="n">
         <v>0</v>
@@ -11823,7 +11843,7 @@
         <v>1115.55</v>
       </c>
       <c r="G255" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H255" s="4" t="n">
         <v>4</v>
@@ -11841,7 +11861,7 @@
         <v>2.55</v>
       </c>
       <c r="M255" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N255" s="4" t="n">
         <v>0</v>
@@ -11867,7 +11887,7 @@
         <v>1115.55</v>
       </c>
       <c r="G256" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H256" s="4" t="n">
         <v>3</v>
@@ -11885,7 +11905,7 @@
         <v>5.385</v>
       </c>
       <c r="M256" s="4" t="n">
-        <v>48.46</v>
+        <v>0</v>
       </c>
       <c r="N256" s="4" t="n">
         <v>0</v>
@@ -11911,7 +11931,7 @@
         <v>1115.55</v>
       </c>
       <c r="G257" s="4" t="n">
-        <v>9</v>
+        <v>2.07</v>
       </c>
       <c r="H257" s="4" t="n">
         <v>1</v>
@@ -11929,7 +11949,7 @@
         <v>9.257</v>
       </c>
       <c r="M257" s="4" t="n">
-        <v>83.31999999999999</v>
+        <v>19.19</v>
       </c>
       <c r="N257" s="4" t="n">
         <v>0</v>
@@ -12307,7 +12327,7 @@
         <v>1115.03</v>
       </c>
       <c r="G266" s="4" t="n">
-        <v>2.03</v>
+        <v>0.4</v>
       </c>
       <c r="H266" s="4" t="n">
         <v>1</v>
@@ -12325,7 +12345,7 @@
         <v>3.599</v>
       </c>
       <c r="M266" s="4" t="n">
-        <v>7.29</v>
+        <v>1.43</v>
       </c>
       <c r="N266" s="4" t="n">
         <v>0</v>
@@ -12351,7 +12371,7 @@
         <v>1121.17</v>
       </c>
       <c r="G267" s="4" t="n">
-        <v>7.58</v>
+        <v>0</v>
       </c>
       <c r="H267" s="4" t="n">
         <v>3</v>
@@ -12369,7 +12389,7 @@
         <v>3.956</v>
       </c>
       <c r="M267" s="4" t="n">
-        <v>29.99</v>
+        <v>0</v>
       </c>
       <c r="N267" s="4" t="n">
         <v>0</v>
@@ -12483,7 +12503,7 @@
         <v>1115.55</v>
       </c>
       <c r="G270" s="4" t="n">
-        <v>5.94</v>
+        <v>0</v>
       </c>
       <c r="H270" s="4" t="n">
         <v>4</v>
@@ -12501,7 +12521,7 @@
         <v>2.55</v>
       </c>
       <c r="M270" s="4" t="n">
-        <v>15.15</v>
+        <v>0</v>
       </c>
       <c r="N270" s="4" t="n">
         <v>0</v>
@@ -12527,7 +12547,7 @@
         <v>1115.55</v>
       </c>
       <c r="G271" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H271" s="4" t="n">
         <v>4</v>
@@ -12545,7 +12565,7 @@
         <v>2.55</v>
       </c>
       <c r="M271" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N271" s="4" t="n">
         <v>0</v>
@@ -12571,7 +12591,7 @@
         <v>1115.55</v>
       </c>
       <c r="G272" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H272" s="4" t="n">
         <v>4</v>
@@ -12589,7 +12609,7 @@
         <v>2.55</v>
       </c>
       <c r="M272" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N272" s="4" t="n">
         <v>0</v>
@@ -12615,7 +12635,7 @@
         <v>1115.55</v>
       </c>
       <c r="G273" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H273" s="4" t="n">
         <v>4</v>
@@ -12633,7 +12653,7 @@
         <v>2.55</v>
       </c>
       <c r="M273" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N273" s="4" t="n">
         <v>0</v>
@@ -12659,7 +12679,7 @@
         <v>1115.55</v>
       </c>
       <c r="G274" s="4" t="n">
-        <v>9</v>
+        <v>0.27</v>
       </c>
       <c r="H274" s="4" t="n">
         <v>2</v>
@@ -12677,7 +12697,7 @@
         <v>5.216</v>
       </c>
       <c r="M274" s="4" t="n">
-        <v>46.95</v>
+        <v>1.39</v>
       </c>
       <c r="N274" s="4" t="n">
         <v>0</v>
@@ -12703,7 +12723,7 @@
         <v>1119.49</v>
       </c>
       <c r="G275" t="n">
-        <v>9</v>
+        <v>8.75</v>
       </c>
       <c r="H275" t="n">
         <v>0</v>
@@ -12721,7 +12741,7 @@
         <v>8.475</v>
       </c>
       <c r="M275" t="n">
-        <v>76.28</v>
+        <v>74.19</v>
       </c>
       <c r="N275" t="n">
         <v>0</v>
@@ -13055,7 +13075,7 @@
         <v>1115.78</v>
       </c>
       <c r="G283" t="n">
-        <v>2.93</v>
+        <v>1.3</v>
       </c>
       <c r="H283" t="n">
         <v>0</v>
@@ -13073,7 +13093,7 @@
         <v>5.092</v>
       </c>
       <c r="M283" t="n">
-        <v>14.94</v>
+        <v>6.64</v>
       </c>
       <c r="N283" t="n">
         <v>0</v>
@@ -13099,7 +13119,7 @@
         <v>1120.38</v>
       </c>
       <c r="G284" s="4" t="n">
-        <v>8.949999999999999</v>
+        <v>0</v>
       </c>
       <c r="H284" s="4" t="n">
         <v>2</v>
@@ -13117,7 +13137,7 @@
         <v>5.164</v>
       </c>
       <c r="M284" s="4" t="n">
-        <v>46.23</v>
+        <v>0</v>
       </c>
       <c r="N284" s="4" t="n">
         <v>0</v>
@@ -13143,7 +13163,7 @@
         <v>1115.55</v>
       </c>
       <c r="G285" s="4" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="H285" s="4" t="n">
         <v>4</v>
@@ -13161,7 +13181,7 @@
         <v>2.55</v>
       </c>
       <c r="M285" s="4" t="n">
-        <v>1.53</v>
+        <v>0</v>
       </c>
       <c r="N285" s="4" t="n">
         <v>0</v>
@@ -13231,7 +13251,7 @@
         <v>1115.55</v>
       </c>
       <c r="G287" s="4" t="n">
-        <v>3.96</v>
+        <v>0</v>
       </c>
       <c r="H287" s="4" t="n">
         <v>4</v>
@@ -13249,7 +13269,7 @@
         <v>2.55</v>
       </c>
       <c r="M287" s="4" t="n">
-        <v>10.1</v>
+        <v>0</v>
       </c>
       <c r="N287" s="4" t="n">
         <v>0</v>
@@ -13275,7 +13295,7 @@
         <v>1115.55</v>
       </c>
       <c r="G288" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H288" s="4" t="n">
         <v>4</v>
@@ -13293,7 +13313,7 @@
         <v>2.55</v>
       </c>
       <c r="M288" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N288" s="4" t="n">
         <v>0</v>
@@ -13319,7 +13339,7 @@
         <v>1115.55</v>
       </c>
       <c r="G289" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H289" s="4" t="n">
         <v>4</v>
@@ -13337,7 +13357,7 @@
         <v>2.55</v>
       </c>
       <c r="M289" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N289" s="4" t="n">
         <v>0</v>
@@ -13363,7 +13383,7 @@
         <v>1115.55</v>
       </c>
       <c r="G290" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H290" s="4" t="n">
         <v>4</v>
@@ -13381,7 +13401,7 @@
         <v>2.55</v>
       </c>
       <c r="M290" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N290" s="4" t="n">
         <v>0</v>
@@ -13407,7 +13427,7 @@
         <v>1115.55</v>
       </c>
       <c r="G291" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H291" s="4" t="n">
         <v>2</v>
@@ -13425,7 +13445,7 @@
         <v>4.5</v>
       </c>
       <c r="M291" s="4" t="n">
-        <v>40.5</v>
+        <v>0</v>
       </c>
       <c r="N291" s="4" t="n">
         <v>0</v>
@@ -13451,7 +13471,7 @@
         <v>1119.41</v>
       </c>
       <c r="G292" t="n">
-        <v>9</v>
+        <v>6.97</v>
       </c>
       <c r="H292" t="n">
         <v>0</v>
@@ -13469,7 +13489,7 @@
         <v>7.818</v>
       </c>
       <c r="M292" t="n">
-        <v>70.36</v>
+        <v>54.48</v>
       </c>
       <c r="N292" t="n">
         <v>0</v>
@@ -13759,7 +13779,7 @@
         <v>1114.7</v>
       </c>
       <c r="G299" t="n">
-        <v>1.08</v>
+        <v>1.01</v>
       </c>
       <c r="H299" t="n">
         <v>0</v>
@@ -13777,7 +13797,7 @@
         <v>4.505</v>
       </c>
       <c r="M299" t="n">
-        <v>4.87</v>
+        <v>4.56</v>
       </c>
       <c r="N299" t="n">
         <v>0</v>
@@ -13803,7 +13823,7 @@
         <v>1119.16</v>
       </c>
       <c r="G300" s="4" t="n">
-        <v>9</v>
+        <v>0.61</v>
       </c>
       <c r="H300" s="4" t="n">
         <v>2</v>
@@ -13821,7 +13841,7 @@
         <v>4.66</v>
       </c>
       <c r="M300" s="4" t="n">
-        <v>41.94</v>
+        <v>2.83</v>
       </c>
       <c r="N300" s="4" t="n">
         <v>0</v>
@@ -13847,7 +13867,7 @@
         <v>1115.55</v>
       </c>
       <c r="G301" s="4" t="n">
-        <v>2.53</v>
+        <v>0</v>
       </c>
       <c r="H301" s="4" t="n">
         <v>4</v>
@@ -13865,7 +13885,7 @@
         <v>2.55</v>
       </c>
       <c r="M301" s="4" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="N301" s="4" t="n">
         <v>0</v>
@@ -13935,7 +13955,7 @@
         <v>1115.55</v>
       </c>
       <c r="G303" s="4" t="n">
-        <v>1.98</v>
+        <v>0</v>
       </c>
       <c r="H303" s="4" t="n">
         <v>4</v>
@@ -13953,7 +13973,7 @@
         <v>2.55</v>
       </c>
       <c r="M303" s="4" t="n">
-        <v>5.05</v>
+        <v>0</v>
       </c>
       <c r="N303" s="4" t="n">
         <v>0</v>
@@ -13979,7 +13999,7 @@
         <v>1115.55</v>
       </c>
       <c r="G304" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H304" s="4" t="n">
         <v>4</v>
@@ -13997,7 +14017,7 @@
         <v>2.55</v>
       </c>
       <c r="M304" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N304" s="4" t="n">
         <v>0</v>
@@ -14023,7 +14043,7 @@
         <v>1115.55</v>
       </c>
       <c r="G305" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H305" s="4" t="n">
         <v>4</v>
@@ -14041,7 +14061,7 @@
         <v>2.55</v>
       </c>
       <c r="M305" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N305" s="4" t="n">
         <v>0</v>
@@ -14067,7 +14087,7 @@
         <v>1115.55</v>
       </c>
       <c r="G306" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H306" s="4" t="n">
         <v>4</v>
@@ -14085,7 +14105,7 @@
         <v>2.55</v>
       </c>
       <c r="M306" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N306" s="4" t="n">
         <v>0</v>
@@ -14111,7 +14131,7 @@
         <v>1115.55</v>
       </c>
       <c r="G307" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H307" s="4" t="n">
         <v>2</v>
@@ -14129,7 +14149,7 @@
         <v>4.399</v>
       </c>
       <c r="M307" s="4" t="n">
-        <v>39.59</v>
+        <v>0</v>
       </c>
       <c r="N307" s="4" t="n">
         <v>0</v>
@@ -14155,7 +14175,7 @@
         <v>1119.09</v>
       </c>
       <c r="G308" t="n">
-        <v>9</v>
+        <v>4.92</v>
       </c>
       <c r="H308" t="n">
         <v>0</v>
@@ -14173,7 +14193,7 @@
         <v>7.864</v>
       </c>
       <c r="M308" t="n">
-        <v>70.78</v>
+        <v>38.67</v>
       </c>
       <c r="N308" t="n">
         <v>0</v>
@@ -14507,7 +14527,7 @@
         <v>1117.93</v>
       </c>
       <c r="G316" s="4" t="n">
-        <v>8.220000000000001</v>
+        <v>1.93</v>
       </c>
       <c r="H316" s="4" t="n">
         <v>2</v>
@@ -14525,7 +14545,7 @@
         <v>4.048</v>
       </c>
       <c r="M316" s="4" t="n">
-        <v>33.29</v>
+        <v>7.82</v>
       </c>
       <c r="N316" s="4" t="n">
         <v>0</v>
@@ -14551,7 +14571,7 @@
         <v>1115.55</v>
       </c>
       <c r="G317" s="4" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="H317" s="4" t="n">
         <v>4</v>
@@ -14569,7 +14589,7 @@
         <v>2.55</v>
       </c>
       <c r="M317" s="4" t="n">
-        <v>11.47</v>
+        <v>0</v>
       </c>
       <c r="N317" s="4" t="n">
         <v>0</v>
@@ -14639,7 +14659,7 @@
         <v>1115.55</v>
       </c>
       <c r="G319" s="4" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="H319" s="4" t="n">
         <v>4</v>
@@ -14657,7 +14677,7 @@
         <v>2.55</v>
       </c>
       <c r="M319" s="4" t="n">
-        <v>0.63</v>
+        <v>0</v>
       </c>
       <c r="N319" s="4" t="n">
         <v>0</v>
@@ -14683,7 +14703,7 @@
         <v>1115.55</v>
       </c>
       <c r="G320" s="4" t="n">
-        <v>8.75</v>
+        <v>0</v>
       </c>
       <c r="H320" s="4" t="n">
         <v>4</v>
@@ -14701,7 +14721,7 @@
         <v>2.55</v>
       </c>
       <c r="M320" s="4" t="n">
-        <v>22.32</v>
+        <v>0</v>
       </c>
       <c r="N320" s="4" t="n">
         <v>0</v>
@@ -14727,7 +14747,7 @@
         <v>1115.55</v>
       </c>
       <c r="G321" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H321" s="4" t="n">
         <v>4</v>
@@ -14745,7 +14765,7 @@
         <v>2.55</v>
       </c>
       <c r="M321" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N321" s="4" t="n">
         <v>0</v>
@@ -14771,7 +14791,7 @@
         <v>1115.55</v>
       </c>
       <c r="G322" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H322" s="4" t="n">
         <v>4</v>
@@ -14789,7 +14809,7 @@
         <v>2.55</v>
       </c>
       <c r="M322" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N322" s="4" t="n">
         <v>0</v>
@@ -14815,7 +14835,7 @@
         <v>1115.55</v>
       </c>
       <c r="G323" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H323" s="4" t="n">
         <v>2</v>
@@ -14833,7 +14853,7 @@
         <v>4.281</v>
       </c>
       <c r="M323" s="4" t="n">
-        <v>38.53</v>
+        <v>0</v>
       </c>
       <c r="N323" s="4" t="n">
         <v>0</v>
@@ -14859,7 +14879,7 @@
         <v>1118.94</v>
       </c>
       <c r="G324" t="n">
-        <v>9</v>
+        <v>2.86</v>
       </c>
       <c r="H324" t="n">
         <v>0</v>
@@ -14877,7 +14897,7 @@
         <v>7.213</v>
       </c>
       <c r="M324" t="n">
-        <v>64.92</v>
+        <v>20.66</v>
       </c>
       <c r="N324" t="n">
         <v>0</v>
@@ -15211,7 +15231,7 @@
         <v>1117.26</v>
       </c>
       <c r="G332" s="4" t="n">
-        <v>6.38</v>
+        <v>2.25</v>
       </c>
       <c r="H332" s="4" t="n">
         <v>2</v>
@@ -15229,7 +15249,7 @@
         <v>3.573</v>
       </c>
       <c r="M332" s="4" t="n">
-        <v>22.79</v>
+        <v>8.06</v>
       </c>
       <c r="N332" s="4" t="n">
         <v>0</v>
@@ -15255,7 +15275,7 @@
         <v>1115.55</v>
       </c>
       <c r="G333" s="4" t="n">
-        <v>6.47</v>
+        <v>0</v>
       </c>
       <c r="H333" s="4" t="n">
         <v>4</v>
@@ -15273,7 +15293,7 @@
         <v>2.55</v>
       </c>
       <c r="M333" s="4" t="n">
-        <v>16.5</v>
+        <v>0</v>
       </c>
       <c r="N333" s="4" t="n">
         <v>0</v>
@@ -15387,7 +15407,7 @@
         <v>1115.55</v>
       </c>
       <c r="G336" s="4" t="n">
-        <v>7.02</v>
+        <v>0</v>
       </c>
       <c r="H336" s="4" t="n">
         <v>4</v>
@@ -15405,7 +15425,7 @@
         <v>2.55</v>
       </c>
       <c r="M336" s="4" t="n">
-        <v>17.91</v>
+        <v>0</v>
       </c>
       <c r="N336" s="4" t="n">
         <v>0</v>
@@ -15431,7 +15451,7 @@
         <v>1115.55</v>
       </c>
       <c r="G337" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H337" s="4" t="n">
         <v>4</v>
@@ -15449,7 +15469,7 @@
         <v>2.55</v>
       </c>
       <c r="M337" s="4" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="N337" s="4" t="n">
         <v>0</v>
@@ -15475,7 +15495,7 @@
         <v>1115.55</v>
       </c>
       <c r="G338" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H338" s="4" t="n">
         <v>3</v>
@@ -15493,7 +15513,7 @@
         <v>2.985</v>
       </c>
       <c r="M338" s="4" t="n">
-        <v>26.87</v>
+        <v>0</v>
       </c>
       <c r="N338" s="4" t="n">
         <v>0</v>
@@ -15519,7 +15539,7 @@
         <v>1117.29</v>
       </c>
       <c r="G339" s="4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H339" s="4" t="n">
         <v>1</v>
@@ -15537,7 +15557,7 @@
         <v>4.663</v>
       </c>
       <c r="M339" s="4" t="n">
-        <v>41.97</v>
+        <v>0</v>
       </c>
       <c r="N339" s="4" t="n">
         <v>0</v>
@@ -15563,7 +15583,7 @@
         <v>1118.87</v>
       </c>
       <c r="G340" t="n">
-        <v>9</v>
+        <v>0.82</v>
       </c>
       <c r="H340" t="n">
         <v>0</v>
@@ -15581,7 +15601,7 @@
         <v>6.624</v>
       </c>
       <c r="M340" t="n">
-        <v>59.62</v>
+        <v>5.46</v>
       </c>
       <c r="N340" t="n">
         <v>0</v>
@@ -15607,7 +15627,7 @@
         <v>1120.25</v>
       </c>
       <c r="G341" t="n">
-        <v>9</v>
+        <v>8.99</v>
       </c>
       <c r="H341" t="n">
         <v>0</v>
@@ -15625,7 +15645,7 @@
         <v>8.504</v>
       </c>
       <c r="M341" t="n">
-        <v>76.54000000000001</v>
+        <v>76.44</v>
       </c>
       <c r="N341" t="n">
         <v>0</v>
@@ -15871,7 +15891,7 @@
         <v>1117.7</v>
       </c>
       <c r="G347" s="4" t="n">
-        <v>2.12</v>
+        <v>0.95</v>
       </c>
       <c r="H347" s="4" t="n">
         <v>1</v>
@@ -15889,7 +15909,7 @@
         <v>3.743</v>
       </c>
       <c r="M347" s="4" t="n">
-        <v>7.95</v>
+        <v>3.54</v>
       </c>
       <c r="N347" s="4" t="n">
         <v>0</v>
@@ -15915,7 +15935,7 @@
         <v>1116.46</v>
       </c>
       <c r="G348" s="4" t="n">
-        <v>7.96</v>
+        <v>0</v>
       </c>
       <c r="H348" s="4" t="n">
         <v>2</v>
@@ -15933,7 +15953,7 @@
         <v>3.069</v>
       </c>
       <c r="M348" s="4" t="n">
-        <v>24.43</v>
+        <v>0</v>
       </c>
       <c r="N348" s="4" t="n">
         <v>0</v>
@@ -15959,7 +15979,7 @@
         <v>1116.71</v>
       </c>
       <c r="G349" s="4" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="H349" s="4" t="n">
         <v>2</v>
@@ -15977,7 +15997,7 @@
         <v>3.115</v>
       </c>
       <c r="M349" s="4" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="N349" s="4" t="n">
         <v>0</v>
@@ -16047,7 +16067,7 @@
         <v>1116.15</v>
       </c>
       <c r="G351" s="4" t="n">
-        <v>4.21</v>
+        <v>0</v>
       </c>
       <c r="H351" s="4" t="n">
         <v>2</v>
@@ -16065,7 +16085,7 @@
         <v>3.325</v>
       </c>
       <c r="M351" s="4" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="N351" s="4" t="n">
         <v>0</v>
@@ -16091,7 +16111,7 @@
         <v>1118.05</v>
       </c>
       <c r="G352" s="4" t="n">
-        <v>8.369999999999999</v>
+        <v>1.21</v>
       </c>
       <c r="H352" s="4" t="n">
         <v>2</v>
@@ -16109,7 +16129,7 @@
         <v>4.062</v>
       </c>
       <c r="M352" s="4" t="n">
-        <v>34.02</v>
+        <v>4.92</v>
       </c>
       <c r="N352" s="4" t="n">
         <v>0</v>
@@ -16135,7 +16155,7 @@
         <v>1119.1</v>
       </c>
       <c r="G353" s="4" t="n">
-        <v>8.83</v>
+        <v>3.32</v>
       </c>
       <c r="H353" s="4" t="n">
         <v>1</v>
@@ -16153,7 +16173,7 @@
         <v>4.744</v>
       </c>
       <c r="M353" s="4" t="n">
-        <v>41.9</v>
+        <v>15.74</v>
       </c>
       <c r="N353" s="4" t="n">
         <v>0</v>
@@ -16179,7 +16199,7 @@
         <v>1119.04</v>
       </c>
       <c r="G354" t="n">
-        <v>9</v>
+        <v>5.34</v>
       </c>
       <c r="H354" t="n">
         <v>0</v>
@@ -16197,7 +16217,7 @@
         <v>5.827</v>
       </c>
       <c r="M354" t="n">
-        <v>52.45</v>
+        <v>31.12</v>
       </c>
       <c r="N354" t="n">
         <v>0</v>
@@ -16223,7 +16243,7 @@
         <v>1120.11</v>
       </c>
       <c r="G355" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
       <c r="H355" t="n">
         <v>0</v>
@@ -16241,7 +16261,7 @@
         <v>6.959</v>
       </c>
       <c r="M355" t="n">
-        <v>62.63</v>
+        <v>50.07</v>
       </c>
       <c r="N355" t="n">
         <v>0</v>
@@ -16267,7 +16287,7 @@
         <v>1120.61</v>
       </c>
       <c r="G356" t="n">
-        <v>9</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="H356" t="n">
         <v>0</v>
@@ -16285,7 +16305,7 @@
         <v>8.503</v>
       </c>
       <c r="M356" t="n">
-        <v>76.53</v>
+        <v>76.28</v>
       </c>
       <c r="N356" t="n">
         <v>0</v>
@@ -16487,7 +16507,7 @@
         <v>1118.13</v>
       </c>
       <c r="G361" t="n">
-        <v>1.97</v>
+        <v>0</v>
       </c>
       <c r="H361" t="n">
         <v>0</v>
@@ -16505,7 +16525,7 @@
         <v>4.422</v>
       </c>
       <c r="M361" t="n">
-        <v>8.699999999999999</v>
+        <v>0</v>
       </c>
       <c r="N361" t="n">
         <v>0</v>
@@ -16531,7 +16551,7 @@
         <v>1118.38</v>
       </c>
       <c r="G362" t="n">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="H362" t="n">
         <v>0</v>
@@ -16549,7 +16569,7 @@
         <v>4.635</v>
       </c>
       <c r="M362" t="n">
-        <v>1.01</v>
+        <v>0</v>
       </c>
       <c r="N362" t="n">
         <v>0</v>
@@ -17056,7 +17076,7 @@
         </is>
       </c>
       <c r="B376" t="n">
-        <v>15794.1</v>
+        <v>12976.86</v>
       </c>
     </row>
     <row r="377">
@@ -17066,7 +17086,7 @@
         </is>
       </c>
       <c r="B377" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="378">
@@ -17076,7 +17096,7 @@
         </is>
       </c>
       <c r="B378" t="n">
-        <v>2581.02</v>
+        <v>1690.92</v>
       </c>
     </row>
     <row r="379">
@@ -17096,7 +17116,7 @@
         </is>
       </c>
       <c r="B380" t="n">
-        <v>1119.119</v>
+        <v>1120.674</v>
       </c>
     </row>
     <row r="381">

</xml_diff>

<commit_message>
Exclude guard room (+1 m all round) as well
The guard room is not drawn in this DXF; its outline comes from the four
Survey.td2 points at its corners. Rooms are now labelled bathroom,
cafeteria and guard room on the plan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/average_levels_1113.xlsx
+++ b/average_levels_1113.xlsx
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1561.63</v>
+        <v>1510.91</v>
       </c>
     </row>
     <row r="4">
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11923.89</v>
+        <v>11508.46</v>
       </c>
     </row>
     <row r="5">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11923.8</v>
+        <v>11508.37</v>
       </c>
     </row>
     <row r="7">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="8">
@@ -570,11 +570,11 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Rooms (bathroom / canteen) + 1 m area excluded (m²)</t>
+          <t>Rooms (bathroom, cafeteria, guard room) + 1 m area excluded (m²)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>129.29</v>
+        <v>180.02</v>
       </c>
     </row>
     <row r="13">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1390.16</v>
+        <v>1440.88</v>
       </c>
     </row>
     <row r="14">
@@ -6221,7 +6221,7 @@
         <v>1120.79</v>
       </c>
       <c r="G127" t="n">
-        <v>9</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="H127" t="n">
         <v>0</v>
@@ -6239,7 +6239,7 @@
         <v>7.717</v>
       </c>
       <c r="M127" t="n">
-        <v>69.45</v>
+        <v>67.84</v>
       </c>
       <c r="N127" t="n">
         <v>0</v>
@@ -6265,7 +6265,7 @@
         <v>1121</v>
       </c>
       <c r="G128" t="n">
-        <v>9</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="H128" t="n">
         <v>0</v>
@@ -6283,7 +6283,7 @@
         <v>7.943</v>
       </c>
       <c r="M128" t="n">
-        <v>71.48999999999999</v>
+        <v>70.48</v>
       </c>
       <c r="N128" t="n">
         <v>0</v>
@@ -7013,7 +7013,7 @@
         <v>1119.65</v>
       </c>
       <c r="G145" t="n">
-        <v>9</v>
+        <v>7.53</v>
       </c>
       <c r="H145" t="n">
         <v>0</v>
@@ -7031,7 +7031,7 @@
         <v>7.179</v>
       </c>
       <c r="M145" t="n">
-        <v>64.61</v>
+        <v>54.08</v>
       </c>
       <c r="N145" t="n">
         <v>0</v>
@@ -7057,7 +7057,7 @@
         <v>1121.67</v>
       </c>
       <c r="G146" s="5" t="n">
-        <v>9</v>
+        <v>0.39</v>
       </c>
       <c r="H146" s="5" t="n">
         <v>0</v>
@@ -7075,7 +7075,7 @@
         <v>8.054</v>
       </c>
       <c r="M146" s="5" t="n">
-        <v>72.48</v>
+        <v>3.14</v>
       </c>
       <c r="N146" s="5" t="n">
         <v>0</v>
@@ -7101,7 +7101,7 @@
         <v>1121.17</v>
       </c>
       <c r="G147" s="5" t="n">
-        <v>9</v>
+        <v>0.01</v>
       </c>
       <c r="H147" s="5" t="n">
         <v>0</v>
@@ -7119,7 +7119,7 @@
         <v>8.004</v>
       </c>
       <c r="M147" s="5" t="n">
-        <v>72.04000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="N147" s="5" t="n">
         <v>0</v>
@@ -7145,7 +7145,7 @@
         <v>1121.05</v>
       </c>
       <c r="G148" t="n">
-        <v>9</v>
+        <v>7.09</v>
       </c>
       <c r="H148" t="n">
         <v>0</v>
@@ -7163,7 +7163,7 @@
         <v>8.063000000000001</v>
       </c>
       <c r="M148" t="n">
-        <v>72.56999999999999</v>
+        <v>57.13</v>
       </c>
       <c r="N148" t="n">
         <v>0</v>
@@ -7893,7 +7893,7 @@
         <v>1119.13</v>
       </c>
       <c r="G165" t="n">
-        <v>9</v>
+        <v>7.08</v>
       </c>
       <c r="H165" t="n">
         <v>0</v>
@@ -7911,7 +7911,7 @@
         <v>7.488</v>
       </c>
       <c r="M165" t="n">
-        <v>67.39</v>
+        <v>53.04</v>
       </c>
       <c r="N165" t="n">
         <v>0</v>
@@ -7937,7 +7937,7 @@
         <v>1121.51</v>
       </c>
       <c r="G166" s="5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H166" s="5" t="n">
         <v>0</v>
@@ -7955,7 +7955,7 @@
         <v>8.496</v>
       </c>
       <c r="M166" s="5" t="n">
-        <v>76.45999999999999</v>
+        <v>0</v>
       </c>
       <c r="N166" s="5" t="n">
         <v>0</v>
@@ -7981,7 +7981,7 @@
         <v>1121.63</v>
       </c>
       <c r="G167" s="5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H167" s="5" t="n">
         <v>0</v>
@@ -7999,7 +7999,7 @@
         <v>8.331</v>
       </c>
       <c r="M167" s="5" t="n">
-        <v>74.98</v>
+        <v>0</v>
       </c>
       <c r="N167" s="5" t="n">
         <v>0</v>
@@ -8025,7 +8025,7 @@
         <v>1121.47</v>
       </c>
       <c r="G168" t="n">
-        <v>9</v>
+        <v>7.31</v>
       </c>
       <c r="H168" t="n">
         <v>0</v>
@@ -8043,7 +8043,7 @@
         <v>8.27</v>
       </c>
       <c r="M168" t="n">
-        <v>74.43000000000001</v>
+        <v>60.44</v>
       </c>
       <c r="N168" t="n">
         <v>0</v>
@@ -8773,7 +8773,7 @@
         <v>1118.64</v>
       </c>
       <c r="G185" t="n">
-        <v>9</v>
+        <v>8.24</v>
       </c>
       <c r="H185" t="n">
         <v>0</v>
@@ -8791,7 +8791,7 @@
         <v>7.226</v>
       </c>
       <c r="M185" t="n">
-        <v>65.03</v>
+        <v>59.53</v>
       </c>
       <c r="N185" t="n">
         <v>0</v>
@@ -8817,7 +8817,7 @@
         <v>1121.63</v>
       </c>
       <c r="G186" t="n">
-        <v>9</v>
+        <v>5.78</v>
       </c>
       <c r="H186" t="n">
         <v>0</v>
@@ -8835,7 +8835,7 @@
         <v>8.590999999999999</v>
       </c>
       <c r="M186" t="n">
-        <v>77.31999999999999</v>
+        <v>49.65</v>
       </c>
       <c r="N186" t="n">
         <v>0</v>
@@ -8861,7 +8861,7 @@
         <v>1121.6</v>
       </c>
       <c r="G187" t="n">
-        <v>9</v>
+        <v>5.74</v>
       </c>
       <c r="H187" t="n">
         <v>0</v>
@@ -8879,7 +8879,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="M187" t="n">
-        <v>76.95</v>
+        <v>49.11</v>
       </c>
       <c r="N187" t="n">
         <v>0</v>
@@ -8905,7 +8905,7 @@
         <v>1121.5</v>
       </c>
       <c r="G188" t="n">
-        <v>9</v>
+        <v>8.44</v>
       </c>
       <c r="H188" t="n">
         <v>0</v>
@@ -8923,7 +8923,7 @@
         <v>8.446</v>
       </c>
       <c r="M188" t="n">
-        <v>76.01000000000001</v>
+        <v>71.28</v>
       </c>
       <c r="N188" t="n">
         <v>0</v>
@@ -17086,7 +17086,7 @@
         </is>
       </c>
       <c r="B376" t="n">
-        <v>11923.89</v>
+        <v>11508.46</v>
       </c>
     </row>
     <row r="377">
@@ -17106,7 +17106,7 @@
         </is>
       </c>
       <c r="B378" t="n">
-        <v>1561.63</v>
+        <v>1510.91</v>
       </c>
     </row>
     <row r="379">
@@ -17126,7 +17126,7 @@
         </is>
       </c>
       <c r="B380" t="n">
-        <v>1120.635</v>
+        <v>1120.617</v>
       </c>
     </row>
     <row r="381">

</xml_diff>

<commit_message>
Stop excluding the culvert; exclude only hangar and rooms
Area 1 volumes now subtract only the hangar, bathroom, cafeteria and
guard room. The plan drawing is renamed excluded_zones.pdf and no longer
shows the culvert.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/average_levels_1113.xlsx
+++ b/average_levels_1113.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1674.31</v>
+        <v>1676.97</v>
       </c>
     </row>
     <row r="4">
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12176.9</v>
+        <v>12186.29</v>
       </c>
     </row>
     <row r="5">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12176.8</v>
+        <v>12186.19</v>
       </c>
     </row>
     <row r="7">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8">
@@ -550,62 +550,52 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Culvert area excluded (m²)</t>
+          <t>Hangar area excluded (m²)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>370.77</v>
+        <v>1159.25</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Hangar area excluded (m²)</t>
+          <t>Rooms (bathroom, cafeteria, guard room) area excluded (m²)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1159.25</v>
+        <v>115.57</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Rooms (bathroom, cafeteria, guard room) area excluded (m²)</t>
+          <t>Total excluded (overlaps counted once) (m²)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>115.57</v>
+        <v>1274.82</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Total excluded (overlaps counted once) (m²)</t>
+          <t>Level deduction (m)</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>1277.48</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>all ground levels lowered by 0.15</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Level deduction (m)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>all ground levels lowered by 0.15</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
           <t>Hangar area</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Unlabeled grid points under the hangar taken as 1115.55</t>
         </is>
@@ -674,7 +664,7 @@
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Area inside hatch excl. culvert, hangar &amp; rooms (m²)</t>
+          <t>Area inside hatch excl. hangar &amp; rooms (m²)</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
@@ -3153,7 +3143,7 @@
         <v>1115.4</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>0.17</v>
+        <v>0.38</v>
       </c>
       <c r="H57" s="4" t="n">
         <v>2</v>
@@ -3171,7 +3161,7 @@
         <v>1.895</v>
       </c>
       <c r="M57" s="4" t="n">
-        <v>0.32</v>
+        <v>0.72</v>
       </c>
       <c r="N57" s="4" t="n">
         <v>0</v>
@@ -16045,7 +16035,7 @@
         <v>1116.5</v>
       </c>
       <c r="G350" s="4" t="n">
-        <v>0</v>
+        <v>0.72</v>
       </c>
       <c r="H350" s="4" t="n">
         <v>2</v>
@@ -16063,7 +16053,7 @@
         <v>2.824</v>
       </c>
       <c r="M350" s="4" t="n">
-        <v>0</v>
+        <v>2.04</v>
       </c>
       <c r="N350" s="4" t="n">
         <v>0</v>
@@ -16089,7 +16079,7 @@
         <v>1116</v>
       </c>
       <c r="G351" s="4" t="n">
-        <v>0.75</v>
+        <v>1.39</v>
       </c>
       <c r="H351" s="4" t="n">
         <v>2</v>
@@ -16107,7 +16097,7 @@
         <v>3.175</v>
       </c>
       <c r="M351" s="4" t="n">
-        <v>2.38</v>
+        <v>4.41</v>
       </c>
       <c r="N351" s="4" t="n">
         <v>0</v>
@@ -16573,7 +16563,7 @@
         <v>1118.23</v>
       </c>
       <c r="G362" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H362" t="n">
         <v>0</v>
@@ -16591,7 +16581,7 @@
         <v>4.485</v>
       </c>
       <c r="M362" t="n">
-        <v>0.32</v>
+        <v>3.62</v>
       </c>
       <c r="N362" t="n">
         <v>0</v>
@@ -16617,7 +16607,7 @@
         <v>1118.65</v>
       </c>
       <c r="G363" t="n">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="H363" t="n">
         <v>0</v>
@@ -16635,7 +16625,7 @@
         <v>4.562</v>
       </c>
       <c r="M363" t="n">
-        <v>0</v>
+        <v>1.63</v>
       </c>
       <c r="N363" t="n">
         <v>0</v>
@@ -17098,7 +17088,7 @@
         </is>
       </c>
       <c r="B376" t="n">
-        <v>12176.9</v>
+        <v>12186.29</v>
       </c>
     </row>
     <row r="377">
@@ -17118,7 +17108,7 @@
         </is>
       </c>
       <c r="B378" t="n">
-        <v>1674.31</v>
+        <v>1676.97</v>
       </c>
     </row>
     <row r="379">
@@ -17138,7 +17128,7 @@
         </is>
       </c>
       <c r="B380" t="n">
-        <v>1120.273</v>
+        <v>1120.267</v>
       </c>
     </row>
     <row r="381">

</xml_diff>